<commit_message>
Item 16: loss proxy → ≥90 DPD seasoned 90 days (1.68% all / 1.15% ex-FPD), side by side; seasoned-denominator vintage and cohort CSVs+SQL filed; tracker v27
</commit_message>
<xml_diff>
--- a/Prior Responses (outside data room)/Zed Portfolio Yield Analysis_20261027_DRAFT.xlsx
+++ b/Prior Responses (outside data room)/Zed Portfolio Yield Analysis_20261027_DRAFT.xlsx
@@ -14,6 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="loss_rate">'Loss Rate'!$F$14</definedName>
+    <definedName name="loss_rate_xfpd">'Loss Rate'!$I$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -90,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -116,7 +117,6 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -870,7 +870,7 @@
     <row r="23" ht="48" customHeight="1">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Loss rate on originated principal (vintages since January 2026, &gt;15 DPD)</t>
+          <t>Loss rate on originated principal — ≥90 DPD, all accounts</t>
         </is>
       </c>
       <c r="C23" s="18">
@@ -883,25 +883,28 @@
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>See the Loss Rate tab. Principal &gt;15 days past due ÷ seasoned originated principal, vintages January–September 2026, gross of recoveries. The same rate is applied to both periods.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="10" t="inlineStr">
-        <is>
-          <t>Loss on receivables (loss rate × turnover)</t>
-        </is>
-      </c>
-      <c r="B24" s="10" t="n"/>
-      <c r="C24" s="12">
-        <f>C23*C22</f>
-        <v/>
-      </c>
-      <c r="D24" s="10" t="n"/>
-      <c r="E24" s="12">
-        <f>E23*E22</f>
-        <v/>
+          <t>See the Loss Rate tab. Principal 90+ days past due ÷ originated principal on statements whose due date is ≥90 days old, vintages since January 2026, gross of recoveries. The same rate is applied to both periods.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="48" customHeight="1">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Loss rate on originated principal — ≥90 DPD, excluding first-payment defaults</t>
+        </is>
+      </c>
+      <c r="C24" s="18">
+        <f>loss_rate_xfpd</f>
+        <v/>
+      </c>
+      <c r="E24" s="18">
+        <f>loss_rate_xfpd</f>
+        <v/>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>Same measure with first-payment-default accounts (never made a payment; treated as fraud/identity cases rather than credit losses) removed from numerator and denominator.</t>
+        </is>
       </c>
     </row>
     <row r="25"/>
@@ -918,96 +921,147 @@
       <c r="F26" s="8" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="inlineStr">
-        <is>
-          <t>Net yield — all revenue, including interchange</t>
-        </is>
-      </c>
-      <c r="B27" s="10" t="n"/>
-      <c r="C27" s="12">
-        <f>C18-C24</f>
-        <v/>
-      </c>
-      <c r="D27" s="10" t="n"/>
-      <c r="E27" s="12">
-        <f>E18-E24</f>
-        <v/>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Loss on receivables — all accounts (loss rate × turnover)</t>
+        </is>
+      </c>
+      <c r="C27" s="9">
+        <f>C23*C22</f>
+        <v/>
+      </c>
+      <c r="E27" s="9">
+        <f>E23*E22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>Net yield — all revenue, all accounts</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="n"/>
+      <c r="C28" s="12">
+        <f>C18-C27</f>
+        <v/>
+      </c>
+      <c r="D28" s="10" t="n"/>
+      <c r="E28" s="12">
+        <f>E18-E27</f>
+        <v/>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
         <is>
           <t>Before operating, servicing and funding costs.</t>
         </is>
       </c>
     </row>
-    <row r="28"/>
-    <row r="29"/>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Loss on receivables — excluding first-payment defaults</t>
+        </is>
+      </c>
+      <c r="C29" s="9">
+        <f>C24*C22</f>
+        <v/>
+      </c>
+      <c r="E29" s="9">
+        <f>E24*E22</f>
+        <v/>
+      </c>
+    </row>
     <row r="30">
-      <c r="A30" s="7" t="inlineStr">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>Net yield — all revenue, excluding first-payment defaults</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="n"/>
+      <c r="C30" s="12">
+        <f>C18-C29</f>
+        <v/>
+      </c>
+      <c r="D30" s="10" t="n"/>
+      <c r="E30" s="12">
+        <f>E18-E29</f>
+        <v/>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>Credit-loss view: first-payment-default receivables would ordinarily be ineligible under a facility.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31"/>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t>Memo — USD equivalents</t>
         </is>
       </c>
-      <c r="B30" s="8" t="n"/>
-      <c r="C30" s="8" t="n"/>
-      <c r="D30" s="8" t="n"/>
-      <c r="E30" s="8" t="n"/>
-      <c r="F30" s="8" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>PHP per USD</t>
-        </is>
-      </c>
-      <c r="B31" s="19" t="n">
-        <v>55.8</v>
-      </c>
-      <c r="D31" s="19" t="n">
-        <v>55.8</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Average receivables outstanding (USD)</t>
-        </is>
-      </c>
-      <c r="B32" s="5">
-        <f>B6/B31</f>
-        <v/>
-      </c>
-      <c r="D32" s="5">
-        <f>D6/D31</f>
-        <v/>
-      </c>
+      <c r="B32" s="8" t="n"/>
+      <c r="C32" s="8" t="n"/>
+      <c r="D32" s="8" t="n"/>
+      <c r="E32" s="8" t="n"/>
+      <c r="F32" s="8" t="n"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Total revenue (USD)</t>
-        </is>
-      </c>
-      <c r="B33" s="5">
-        <f>B14/B31</f>
-        <v/>
-      </c>
-      <c r="D33" s="5">
-        <f>D14/D31</f>
-        <v/>
+          <t>PHP per USD</t>
+        </is>
+      </c>
+      <c r="B33" s="19" t="n">
+        <v>55.8</v>
+      </c>
+      <c r="D33" s="19" t="n">
+        <v>55.8</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>Average receivables outstanding (USD)</t>
+        </is>
+      </c>
+      <c r="B34" s="5">
+        <f>B6/B33</f>
+        <v/>
+      </c>
+      <c r="D34" s="5">
+        <f>D6/D33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Total revenue (USD)</t>
+        </is>
+      </c>
+      <c r="B35" s="5">
+        <f>B14/B33</f>
+        <v/>
+      </c>
+      <c r="D35" s="5">
+        <f>D14/D33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>Principal originated (USD)</t>
         </is>
       </c>
-      <c r="B34" s="5">
-        <f>B21/B31</f>
-        <v/>
-      </c>
-      <c r="D34" s="5">
-        <f>D21/D31</f>
+      <c r="B36" s="5">
+        <f>B21/B33</f>
+        <v/>
+      </c>
+      <c r="D36" s="5">
+        <f>D21/D33</f>
         <v/>
       </c>
     </row>
@@ -1826,7 +1880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1834,22 +1888,23 @@
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Loss rate on originated principal — vintages since January 2026</t>
+          <t>Loss rate on originated principal — 90+ days past due, vintages since January 2026</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PHP. Each row is the principal originated in that month and how much of it is on an account more than 15 days past due today (data as of 26 October 2026). Vintages begin January 2026, the first full month after the current underwriting model was introduced (December 2025).</t>
+          <t>PHP. Each row is the principal originated in that month and how much of it sits on an account 90 or more days past due today (data as of 27 October 2026). Vintages begin January 2026, the first full month after the current underwriting model was introduced (December 2025).</t>
         </is>
       </c>
     </row>
@@ -1872,27 +1927,32 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Principal on statements ≥16 days past due date (seasoned)</t>
+          <t>Principal on statements ≥90 days past due date (seasoned)</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Principal &gt;15 DPD today</t>
+          <t>Principal ≥90 DPD today</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Loss rate (&gt;15 DPD ÷ seasoned principal)</t>
+          <t>Loss rate — all accounts</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>of which ≥90 DPD</t>
+          <t>Seasoned principal, ex-FPD</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>≥90 DPD as share of &gt;15 DPD</t>
+          <t>Principal ≥90 DPD, ex-FPD</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Loss rate — ex-FPD</t>
         </is>
       </c>
     </row>
@@ -1915,14 +1975,17 @@
         <v>1772322.4</v>
       </c>
       <c r="F5" s="18">
-        <f>E5/D5</f>
+        <f>IF(D5=0,"not yet seasoned",E5/D5)</f>
         <v/>
       </c>
       <c r="G5" s="5" t="n">
-        <v>1772322.4</v>
-      </c>
-      <c r="H5" s="9">
-        <f>IF(E5=0,"",G5/E5)</f>
+        <v>69690793.31</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>1577286.85</v>
+      </c>
+      <c r="I5" s="18">
+        <f>IF(G5=0,"not yet seasoned",H5/G5)</f>
         <v/>
       </c>
     </row>
@@ -1945,14 +2008,17 @@
         <v>716893.6800000001</v>
       </c>
       <c r="F6" s="18">
-        <f>E6/D6</f>
+        <f>IF(D6=0,"not yet seasoned",E6/D6)</f>
         <v/>
       </c>
       <c r="G6" s="5" t="n">
-        <v>716893.6800000001</v>
-      </c>
-      <c r="H6" s="9">
-        <f>IF(E6=0,"",G6/E6)</f>
+        <v>60789404.74</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>685527.14</v>
+      </c>
+      <c r="I6" s="18">
+        <f>IF(G6=0,"not yet seasoned",H6/G6)</f>
         <v/>
       </c>
     </row>
@@ -1975,14 +2041,17 @@
         <v>1967651.07</v>
       </c>
       <c r="F7" s="18">
-        <f>E7/D7</f>
+        <f>IF(D7=0,"not yet seasoned",E7/D7)</f>
         <v/>
       </c>
       <c r="G7" s="5" t="n">
-        <v>1967651.07</v>
-      </c>
-      <c r="H7" s="9">
-        <f>IF(E7=0,"",G7/E7)</f>
+        <v>89089554.73999999</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>1404938.62</v>
+      </c>
+      <c r="I7" s="18">
+        <f>IF(G7=0,"not yet seasoned",H7/G7)</f>
         <v/>
       </c>
     </row>
@@ -2002,17 +2071,20 @@
         <v>107115373.17</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>2422156.56</v>
+        <v>2382018.67</v>
       </c>
       <c r="F8" s="18">
-        <f>E8/D8</f>
+        <f>IF(D8=0,"not yet seasoned",E8/D8)</f>
         <v/>
       </c>
       <c r="G8" s="5" t="n">
-        <v>2382018.67</v>
-      </c>
-      <c r="H8" s="9">
-        <f>IF(E8=0,"",G8/E8)</f>
+        <v>106123235.92</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>1471002.56</v>
+      </c>
+      <c r="I8" s="18">
+        <f>IF(G8=0,"not yet seasoned",H8/G8)</f>
         <v/>
       </c>
     </row>
@@ -2032,17 +2104,20 @@
         <v>118184976.17</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>2191111.12</v>
+        <v>1950748.96</v>
       </c>
       <c r="F9" s="18">
-        <f>E9/D9</f>
+        <f>IF(D9=0,"not yet seasoned",E9/D9)</f>
         <v/>
       </c>
       <c r="G9" s="5" t="n">
-        <v>1950748.96</v>
-      </c>
-      <c r="H9" s="9">
-        <f>IF(E9=0,"",G9/E9)</f>
+        <v>117226741.83</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>1061583</v>
+      </c>
+      <c r="I9" s="18">
+        <f>IF(G9=0,"not yet seasoned",H9/G9)</f>
         <v/>
       </c>
     </row>
@@ -2062,17 +2137,20 @@
         <v>136417479.48</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1666168.59</v>
+        <v>959336.8100000001</v>
       </c>
       <c r="F10" s="18">
-        <f>E10/D10</f>
+        <f>IF(D10=0,"not yet seasoned",E10/D10)</f>
         <v/>
       </c>
       <c r="G10" s="5" t="n">
-        <v>959336.8100000001</v>
-      </c>
-      <c r="H10" s="9">
-        <f>IF(E10=0,"",G10/E10)</f>
+        <v>135917605.98</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>459463.31</v>
+      </c>
+      <c r="I10" s="18">
+        <f>IF(G10=0,"not yet seasoned",H10/G10)</f>
         <v/>
       </c>
     </row>
@@ -2089,20 +2167,23 @@
         <v>140624271.71</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>140624271.71</v>
+        <v>0</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>1456435.12</v>
+        <v>38218.7</v>
       </c>
       <c r="F11" s="18">
-        <f>E11/D11</f>
+        <f>IF(D11=0,"not yet seasoned",E11/D11)</f>
         <v/>
       </c>
       <c r="G11" s="5" t="n">
-        <v>38218.7</v>
-      </c>
-      <c r="H11" s="9">
-        <f>IF(E11=0,"",G11/E11)</f>
+        <v>0</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>8828.190000000001</v>
+      </c>
+      <c r="I11" s="18">
+        <f>IF(G11=0,"not yet seasoned",H11/G11)</f>
         <v/>
       </c>
     </row>
@@ -2119,20 +2200,23 @@
         <v>141888335.14</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>141888335.14</v>
+        <v>0</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>1670573.34</v>
+        <v>0</v>
       </c>
       <c r="F12" s="18">
-        <f>E12/D12</f>
+        <f>IF(D12=0,"not yet seasoned",E12/D12)</f>
         <v/>
       </c>
       <c r="G12" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="9">
-        <f>IF(E12=0,"",G12/E12)</f>
+      <c r="H12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="18">
+        <f>IF(G12=0,"not yet seasoned",H12/G12)</f>
         <v/>
       </c>
     </row>
@@ -2149,20 +2233,23 @@
         <v>160221212.53</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>59316000.94</v>
+        <v>0</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>446581.32</v>
+        <v>0</v>
       </c>
       <c r="F13" s="18">
-        <f>E13/D13</f>
+        <f>IF(D13=0,"not yet seasoned",E13/D13)</f>
         <v/>
       </c>
       <c r="G13" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="9">
-        <f>IF(E13=0,"",G13/E13)</f>
+      <c r="H13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="18">
+        <f>IF(G13=0,"not yet seasoned",H13/G13)</f>
         <v/>
       </c>
     </row>
@@ -2196,81 +2283,78 @@
         <f>SUM(G5:G13)</f>
         <v/>
       </c>
-      <c r="H14" s="21">
-        <f>G14/E14</f>
+      <c r="H14" s="14">
+        <f>SUM(H5:H13)</f>
+        <v/>
+      </c>
+      <c r="I14" s="20">
+        <f>H14/G14</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Vintages January–April 2026 only (six or more months on book)</t>
+          <t>Memo: principal ≥90 DPD on first-payment-default accounts</t>
         </is>
       </c>
       <c r="E15" s="5">
-        <f>SUM(E5:E8)</f>
-        <v/>
-      </c>
-      <c r="G15" s="5">
-        <f>SUM(G5:G8)</f>
-        <v/>
-      </c>
-      <c r="H15" s="9">
-        <f>G15/E15</f>
-        <v/>
+        <f>E14-H14</f>
+        <v/>
+      </c>
+      <c r="F15" s="9">
+        <f>E15/E14</f>
+        <v/>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>share of all ≥90 DPD principal</t>
+        </is>
       </c>
     </row>
     <row r="16"/>
     <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="22" t="inlineStr">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>How to read this table</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="45" customHeight="1">
+    <row r="18" ht="48" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>• Loss measure. We use principal more than 15 days past due as the loss measure. On vintages that are six or more months on book, over 99% of the principal that went &gt;15 DPD is ≥90 DPD today (column H), i.e. almost nothing cures. The ≥90 DPD column cannot be used on its own because the July–September vintages are not yet old enough to reach 90 days past due.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="45" customHeight="1">
+          <t>• Loss measure. Principal on accounts 90 or more days past due is used as the proxy for loss. Zed fully provisions at 180 days past due and has not yet written off any balances, so no recoveries are assumed and nothing has been reduced for cash collected after an account went delinquent. Interest and fees are excluded from both numerator and denominator.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="48" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>• Seasoning. The denominator counts only principal whose statement due date is at least 16 days in the past, so the newest months are not diluted by purchases that cannot yet be delinquent. The September 2026 vintage is therefore partly seasoned and its rate will move as the rest of the month's statements pass their due dates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="45" customHeight="1">
+          <t>• Seasoning. The denominator counts only principal whose statement due date is at least 90 days in the past, so the rate is measured on principal that has had the chance to reach 90 days past due. On this basis the July–September 2026 vintages are not yet measurable and are shown for completeness; the small amount of ≥90 DPD principal attributed to July sits on accounts that went delinquent on earlier statements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="48" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>• Gross of recoveries. Zed fully provisions at 180 days past due and has not yet written off any balances, so no recoveries are assumed. Nothing in this table has been reduced for cash collected after an account went delinquent.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="45" customHeight="1">
+          <t>• First-payment defaults (FPD). An account whose first-ever statement was the one missed, i.e. a cardholder who never made a payment. These are treated as fraud or identity cases rather than credit losses and are shown separately: the ex-FPD columns remove those accounts from both numerator and denominator. Receivables of this kind would ordinarily fall outside facility eligibility criteria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="48" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>• Interest and fees are excluded from both numerator and denominator; this is a loss rate on principal lent.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="45" customHeight="1">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
           <t>• Why January 2026. The current underwriting model (V2) was deployed in December 2025 and is the model that originates the portfolio today; earlier vintages were originated under the prior model.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A18:H18"/>
-    <mergeCell ref="A21:H21"/>
-    <mergeCell ref="A20:H20"/>
-    <mergeCell ref="A19:H19"/>
-    <mergeCell ref="A22:H22"/>
-    <mergeCell ref="A17:H17"/>
+  <mergeCells count="5">
+    <mergeCell ref="A19:I19"/>
+    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="A18:I18"/>
+    <mergeCell ref="A20:I20"/>
+    <mergeCell ref="A21:I21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2310,7 +2394,7 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="23" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>Scope</t>
         </is>
@@ -2322,7 +2406,7 @@
       </c>
     </row>
     <row r="5" ht="60" customHeight="1">
-      <c r="A5" s="23" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>Average receivables</t>
         </is>
@@ -2334,7 +2418,7 @@
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="23" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>Annualization</t>
         </is>
@@ -2346,7 +2430,7 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="23" t="inlineStr">
+      <c r="A7" s="22" t="inlineStr">
         <is>
           <t>Revolving interest</t>
         </is>
@@ -2358,7 +2442,7 @@
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="23" t="inlineStr">
+      <c r="A8" s="22" t="inlineStr">
         <is>
           <t>Installment interest and upfront fees</t>
         </is>
@@ -2370,7 +2454,7 @@
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="23" t="inlineStr">
+      <c r="A9" s="22" t="inlineStr">
         <is>
           <t>Late payment fees</t>
         </is>
@@ -2382,7 +2466,7 @@
       </c>
     </row>
     <row r="10" ht="75" customHeight="1">
-      <c r="A10" s="23" t="inlineStr">
+      <c r="A10" s="22" t="inlineStr">
         <is>
           <t>Interchange</t>
         </is>
@@ -2394,7 +2478,7 @@
       </c>
     </row>
     <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="23" t="inlineStr">
+      <c r="A11" s="22" t="inlineStr">
         <is>
           <t>Principal originated</t>
         </is>
@@ -2405,20 +2489,20 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="75" customHeight="1">
-      <c r="A12" s="23" t="inlineStr">
+    <row r="12" ht="90" customHeight="1">
+      <c r="A12" s="22" t="inlineStr">
         <is>
           <t>Loss rate</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Principal on accounts more than 15 days past due today, divided by originated principal on statements whose due date is at least 16 days old, for origination months January–September 2026. The reasons for the window, the &gt;15 DPD measure and the seasoning rule are set out on the Loss Rate tab. Gross of recoveries; no balances have been written off to date (full provision at 180 DPD).</t>
+          <t>Principal on accounts 90 or more days past due today, divided by originated principal on statements whose due date is at least 90 days old, for origination months January–September 2026 (in practice January–June, the vintages old enough to be measured). Shown for all accounts and excluding first-payment defaults; the window, the seasoning rule and the FPD definition are set out on the Loss Rate tab. Gross of recoveries; no balances have been written off to date (full provision at 180 DPD).</t>
         </is>
       </c>
     </row>
     <row r="13" ht="45" customHeight="1">
-      <c r="A13" s="23" t="inlineStr">
+      <c r="A13" s="22" t="inlineStr">
         <is>
           <t>Loss on receivables</t>
         </is>
@@ -2430,7 +2514,7 @@
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="23" t="inlineStr">
+      <c r="A14" s="22" t="inlineStr">
         <is>
           <t>Net yield</t>
         </is>
@@ -2441,20 +2525,20 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="45" customHeight="1">
-      <c r="A15" s="23" t="inlineStr">
+    <row r="15" ht="60" customHeight="1">
+      <c r="A15" s="22" t="inlineStr">
         <is>
           <t>Sources</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Zed management reporting built from the i2c transaction and settlement extracts (revenue, receivables, purchase volume) and Zed's statement and delinquency data (originations, delinquency by origination month). Data as of 26 October 2026; September 2026 is the latest complete month.</t>
+          <t>Zed management reporting built from the i2c transaction and settlement extracts (revenue, receivables, purchase volume; as of 26 October 2026) and Zed's statement and delinquency data (originations, delinquency by origination month; as of 27 October 2026). September 2026 is the latest complete month.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="23" t="inlineStr">
+      <c r="A16" s="22" t="inlineStr">
         <is>
           <t>Prepared</t>
         </is>

</xml_diff>

<commit_message>
Item 16: present ≥90 DPD ex-FPD only (1.15%, Sep net 23.1%); excluded FPD principal shown; tracker v28
</commit_message>
<xml_diff>
--- a/Prior Responses (outside data room)/Zed Portfolio Yield Analysis_20261027_DRAFT.xlsx
+++ b/Prior Responses (outside data room)/Zed Portfolio Yield Analysis_20261027_DRAFT.xlsx
@@ -13,8 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="loss_rate">'Loss Rate'!$F$14</definedName>
-    <definedName name="loss_rate_xfpd">'Loss Rate'!$I$14</definedName>
+    <definedName name="loss_rate_xfpd">'Loss Rate'!$H$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -488,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -867,201 +866,144 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="48" customHeight="1">
+    <row r="23" ht="64" customHeight="1">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Loss rate on originated principal — ≥90 DPD, all accounts</t>
+          <t>Loss rate on originated principal — ≥90 DPD, excluding first-payment defaults</t>
         </is>
       </c>
       <c r="C23" s="18">
-        <f>loss_rate</f>
+        <f>loss_rate_xfpd</f>
         <v/>
       </c>
       <c r="E23" s="18">
-        <f>loss_rate</f>
+        <f>loss_rate_xfpd</f>
         <v/>
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>See the Loss Rate tab. Principal 90+ days past due ÷ originated principal on statements whose due date is ≥90 days old, vintages since January 2026, gross of recoveries. The same rate is applied to both periods.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="48" customHeight="1">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Loss rate on originated principal — ≥90 DPD, excluding first-payment defaults</t>
-        </is>
-      </c>
-      <c r="C24" s="18">
-        <f>loss_rate_xfpd</f>
-        <v/>
-      </c>
-      <c r="E24" s="18">
-        <f>loss_rate_xfpd</f>
-        <v/>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>Same measure with first-payment-default accounts (never made a payment; treated as fraud/identity cases rather than credit losses) removed from numerator and denominator.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25"/>
+          <t>See the Loss Rate tab. Principal 90+ days past due ÷ originated principal on statements whose due date is ≥90 days old, vintages since January 2026, gross of recoveries; first-payment-default accounts (never made a payment; fraud/identity rather than credit) excluded from numerator and denominator. The same rate is applied to both periods.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24"/>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>Net yield (gross yield less loss on receivables)</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="n"/>
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="8" t="n"/>
+      <c r="E25" s="8" t="n"/>
+      <c r="F25" s="8" t="n"/>
+    </row>
     <row r="26">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>Net yield (gross yield less loss on receivables)</t>
-        </is>
-      </c>
-      <c r="B26" s="8" t="n"/>
-      <c r="C26" s="8" t="n"/>
-      <c r="D26" s="8" t="n"/>
-      <c r="E26" s="8" t="n"/>
-      <c r="F26" s="8" t="n"/>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Loss on receivables (loss rate × turnover)</t>
+        </is>
+      </c>
+      <c r="C26" s="9">
+        <f>C23*C22</f>
+        <v/>
+      </c>
+      <c r="E26" s="9">
+        <f>E23*E22</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Loss on receivables — all accounts (loss rate × turnover)</t>
-        </is>
-      </c>
-      <c r="C27" s="9">
-        <f>C23*C22</f>
-        <v/>
-      </c>
-      <c r="E27" s="9">
-        <f>E23*E22</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="10" t="inlineStr">
-        <is>
-          <t>Net yield — all revenue, all accounts</t>
-        </is>
-      </c>
-      <c r="B28" s="10" t="n"/>
-      <c r="C28" s="12">
-        <f>C18-C27</f>
-        <v/>
-      </c>
-      <c r="D28" s="10" t="n"/>
-      <c r="E28" s="12">
-        <f>E18-E27</f>
-        <v/>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>Net yield — all revenue, including interchange</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="n"/>
+      <c r="C27" s="12">
+        <f>C18-C26</f>
+        <v/>
+      </c>
+      <c r="D27" s="10" t="n"/>
+      <c r="E27" s="12">
+        <f>E18-E26</f>
+        <v/>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
         <is>
           <t>Before operating, servicing and funding costs.</t>
         </is>
       </c>
     </row>
+    <row r="28"/>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Loss on receivables — excluding first-payment defaults</t>
-        </is>
-      </c>
-      <c r="C29" s="9">
-        <f>C24*C22</f>
-        <v/>
-      </c>
-      <c r="E29" s="9">
-        <f>E24*E22</f>
-        <v/>
-      </c>
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>Memo — USD equivalents</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="n"/>
+      <c r="C29" s="8" t="n"/>
+      <c r="D29" s="8" t="n"/>
+      <c r="E29" s="8" t="n"/>
+      <c r="F29" s="8" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="10" t="inlineStr">
-        <is>
-          <t>Net yield — all revenue, excluding first-payment defaults</t>
-        </is>
-      </c>
-      <c r="B30" s="10" t="n"/>
-      <c r="C30" s="12">
-        <f>C18-C29</f>
-        <v/>
-      </c>
-      <c r="D30" s="10" t="n"/>
-      <c r="E30" s="12">
-        <f>E18-E29</f>
-        <v/>
-      </c>
-      <c r="F30" s="6" t="inlineStr">
-        <is>
-          <t>Credit-loss view: first-payment-default receivables would ordinarily be ineligible under a facility.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31"/>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>PHP per USD</t>
+        </is>
+      </c>
+      <c r="B30" s="19" t="n">
+        <v>55.8</v>
+      </c>
+      <c r="D30" s="19" t="n">
+        <v>55.8</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Average receivables outstanding (USD)</t>
+        </is>
+      </c>
+      <c r="B31" s="5">
+        <f>B6/B30</f>
+        <v/>
+      </c>
+      <c r="D31" s="5">
+        <f>D6/D30</f>
+        <v/>
+      </c>
+    </row>
     <row r="32">
-      <c r="A32" s="7" t="inlineStr">
-        <is>
-          <t>Memo — USD equivalents</t>
-        </is>
-      </c>
-      <c r="B32" s="8" t="n"/>
-      <c r="C32" s="8" t="n"/>
-      <c r="D32" s="8" t="n"/>
-      <c r="E32" s="8" t="n"/>
-      <c r="F32" s="8" t="n"/>
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Total revenue (USD)</t>
+        </is>
+      </c>
+      <c r="B32" s="5">
+        <f>B14/B30</f>
+        <v/>
+      </c>
+      <c r="D32" s="5">
+        <f>D14/D30</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>PHP per USD</t>
-        </is>
-      </c>
-      <c r="B33" s="19" t="n">
-        <v>55.8</v>
-      </c>
-      <c r="D33" s="19" t="n">
-        <v>55.8</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Average receivables outstanding (USD)</t>
-        </is>
-      </c>
-      <c r="B34" s="5">
-        <f>B6/B33</f>
-        <v/>
-      </c>
-      <c r="D34" s="5">
-        <f>D6/D33</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Total revenue (USD)</t>
-        </is>
-      </c>
-      <c r="B35" s="5">
-        <f>B14/B33</f>
-        <v/>
-      </c>
-      <c r="D35" s="5">
-        <f>D14/D33</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
           <t>Principal originated (USD)</t>
         </is>
       </c>
-      <c r="B36" s="5">
-        <f>B21/B33</f>
-        <v/>
-      </c>
-      <c r="D36" s="5">
-        <f>D21/D33</f>
+      <c r="B33" s="5">
+        <f>B21/B30</f>
+        <v/>
+      </c>
+      <c r="D33" s="5">
+        <f>D21/D30</f>
         <v/>
       </c>
     </row>
@@ -1880,18 +1822,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1932,27 +1873,22 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Principal ≥90 DPD today</t>
+          <t>Principal ≥90 DPD on first-payment-default accounts (excluded)</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Loss rate — all accounts</t>
+          <t>Seasoned principal, ex-FPD</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Seasoned principal, ex-FPD</t>
+          <t>Principal ≥90 DPD, ex-FPD</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Principal ≥90 DPD, ex-FPD</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>Loss rate — ex-FPD</t>
+          <t>Loss rate (≥90 DPD ex-FPD ÷ seasoned principal ex-FPD)</t>
         </is>
       </c>
     </row>
@@ -1972,20 +1908,16 @@
         <v>69900973.84</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>1772322.4</v>
-      </c>
-      <c r="F5" s="18">
-        <f>IF(D5=0,"not yet seasoned",E5/D5)</f>
-        <v/>
+        <v>195035.55</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>69690793.31</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>69690793.31</v>
-      </c>
-      <c r="H5" s="5" t="n">
         <v>1577286.85</v>
       </c>
-      <c r="I5" s="18">
-        <f>IF(G5=0,"not yet seasoned",H5/G5)</f>
+      <c r="H5" s="18">
+        <f>IF(F5=0,"not yet seasoned",G5/F5)</f>
         <v/>
       </c>
     </row>
@@ -2005,20 +1937,16 @@
         <v>60820771.28</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>716893.6800000001</v>
-      </c>
-      <c r="F6" s="18">
-        <f>IF(D6=0,"not yet seasoned",E6/D6)</f>
-        <v/>
+        <v>31366.54</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>60789404.74</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>60789404.74</v>
-      </c>
-      <c r="H6" s="5" t="n">
         <v>685527.14</v>
       </c>
-      <c r="I6" s="18">
-        <f>IF(G6=0,"not yet seasoned",H6/G6)</f>
+      <c r="H6" s="18">
+        <f>IF(F6=0,"not yet seasoned",G6/F6)</f>
         <v/>
       </c>
     </row>
@@ -2038,20 +1966,16 @@
         <v>89743205.59</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>1967651.07</v>
-      </c>
-      <c r="F7" s="18">
-        <f>IF(D7=0,"not yet seasoned",E7/D7)</f>
-        <v/>
+        <v>562712.45</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>89089554.73999999</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>89089554.73999999</v>
-      </c>
-      <c r="H7" s="5" t="n">
         <v>1404938.62</v>
       </c>
-      <c r="I7" s="18">
-        <f>IF(G7=0,"not yet seasoned",H7/G7)</f>
+      <c r="H7" s="18">
+        <f>IF(F7=0,"not yet seasoned",G7/F7)</f>
         <v/>
       </c>
     </row>
@@ -2071,20 +1995,16 @@
         <v>107115373.17</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>2382018.67</v>
-      </c>
-      <c r="F8" s="18">
-        <f>IF(D8=0,"not yet seasoned",E8/D8)</f>
-        <v/>
+        <v>911016.11</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>106123235.92</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>106123235.92</v>
-      </c>
-      <c r="H8" s="5" t="n">
         <v>1471002.56</v>
       </c>
-      <c r="I8" s="18">
-        <f>IF(G8=0,"not yet seasoned",H8/G8)</f>
+      <c r="H8" s="18">
+        <f>IF(F8=0,"not yet seasoned",G8/F8)</f>
         <v/>
       </c>
     </row>
@@ -2104,20 +2024,16 @@
         <v>118184976.17</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>1950748.96</v>
-      </c>
-      <c r="F9" s="18">
-        <f>IF(D9=0,"not yet seasoned",E9/D9)</f>
-        <v/>
+        <v>889165.96</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>117226741.83</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>117226741.83</v>
-      </c>
-      <c r="H9" s="5" t="n">
         <v>1061583</v>
       </c>
-      <c r="I9" s="18">
-        <f>IF(G9=0,"not yet seasoned",H9/G9)</f>
+      <c r="H9" s="18">
+        <f>IF(F9=0,"not yet seasoned",G9/F9)</f>
         <v/>
       </c>
     </row>
@@ -2137,20 +2053,16 @@
         <v>136417479.48</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>959336.8100000001</v>
-      </c>
-      <c r="F10" s="18">
-        <f>IF(D10=0,"not yet seasoned",E10/D10)</f>
-        <v/>
+        <v>499873.5</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>135917605.98</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>135917605.98</v>
-      </c>
-      <c r="H10" s="5" t="n">
         <v>459463.31</v>
       </c>
-      <c r="I10" s="18">
-        <f>IF(G10=0,"not yet seasoned",H10/G10)</f>
+      <c r="H10" s="18">
+        <f>IF(F10=0,"not yet seasoned",G10/F10)</f>
         <v/>
       </c>
     </row>
@@ -2170,20 +2082,16 @@
         <v>0</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>38218.7</v>
-      </c>
-      <c r="F11" s="18">
-        <f>IF(D11=0,"not yet seasoned",E11/D11)</f>
-        <v/>
+        <v>29390.51</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="5" t="n">
         <v>8828.190000000001</v>
       </c>
-      <c r="I11" s="18">
-        <f>IF(G11=0,"not yet seasoned",H11/G11)</f>
+      <c r="H11" s="18">
+        <f>IF(F11=0,"not yet seasoned",G11/F11)</f>
         <v/>
       </c>
     </row>
@@ -2205,18 +2113,14 @@
       <c r="E12" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="18">
-        <f>IF(D12=0,"not yet seasoned",E12/D12)</f>
-        <v/>
+      <c r="F12" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="G12" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="18">
-        <f>IF(G12=0,"not yet seasoned",H12/G12)</f>
+      <c r="H12" s="18">
+        <f>IF(F12=0,"not yet seasoned",G12/F12)</f>
         <v/>
       </c>
     </row>
@@ -2238,18 +2142,14 @@
       <c r="E13" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="18">
-        <f>IF(D13=0,"not yet seasoned",E13/D13)</f>
-        <v/>
+      <c r="F13" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="G13" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="18">
-        <f>IF(G13=0,"not yet seasoned",H13/G13)</f>
+      <c r="H13" s="18">
+        <f>IF(F13=0,"not yet seasoned",G13/F13)</f>
         <v/>
       </c>
     </row>
@@ -2275,86 +2175,62 @@
         <f>SUM(E5:E13)</f>
         <v/>
       </c>
-      <c r="F14" s="20">
-        <f>E14/D14</f>
+      <c r="F14" s="14">
+        <f>SUM(F5:F13)</f>
         <v/>
       </c>
       <c r="G14" s="14">
         <f>SUM(G5:G13)</f>
         <v/>
       </c>
-      <c r="H14" s="14">
-        <f>SUM(H5:H13)</f>
-        <v/>
-      </c>
-      <c r="I14" s="20">
-        <f>H14/G14</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Memo: principal ≥90 DPD on first-payment-default accounts</t>
-        </is>
-      </c>
-      <c r="E15" s="5">
-        <f>E14-H14</f>
-        <v/>
-      </c>
-      <c r="F15" s="9">
-        <f>E15/E14</f>
-        <v/>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>share of all ≥90 DPD principal</t>
-        </is>
-      </c>
-    </row>
-    <row r="16"/>
-    <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="H14" s="20">
+        <f>G14/F14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15"/>
+    <row r="16" ht="15" customHeight="1">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>How to read this table</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>• Loss measure. Principal on accounts 90 or more days past due is used as the proxy for loss. Zed fully provisions at 180 days past due and has not yet written off any balances, so no recoveries are assumed and nothing has been reduced for cash collected after an account went delinquent. Interest and fees are excluded from both numerator and denominator.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="48" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>• Loss measure. Principal on accounts 90 or more days past due is used as the proxy for loss. Zed fully provisions at 180 days past due and has not yet written off any balances, so no recoveries are assumed and nothing has been reduced for cash collected after an account went delinquent. Interest and fees are excluded from both numerator and denominator.</t>
+          <t>• Seasoning. The denominator counts only principal whose statement due date is at least 90 days in the past, so the rate is measured on principal that has had the chance to reach 90 days past due. On this basis the July–September 2026 vintages are not yet measurable and are shown for completeness.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="48" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>• Seasoning. The denominator counts only principal whose statement due date is at least 90 days in the past, so the rate is measured on principal that has had the chance to reach 90 days past due. On this basis the July–September 2026 vintages are not yet measurable and are shown for completeness; the small amount of ≥90 DPD principal attributed to July sits on accounts that went delinquent on earlier statements.</t>
+          <t>• First-payment defaults (FPD). An account whose first-ever statement was the one missed, i.e. a cardholder who never made a payment. These are fraud or identity cases rather than credit losses and are excluded from the loss rate; the principal excluded is shown in column E so the adjustment is visible. Receivables of this kind would ordinarily fall outside facility eligibility criteria. Zed now manages first-payment default through dedicated onboarding and fraud controls, separately from credit underwriting.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="48" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>• First-payment defaults (FPD). An account whose first-ever statement was the one missed, i.e. a cardholder who never made a payment. These are treated as fraud or identity cases rather than credit losses and are shown separately: the ex-FPD columns remove those accounts from both numerator and denominator. Receivables of this kind would ordinarily fall outside facility eligibility criteria.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="48" customHeight="1">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
           <t>• Why January 2026. The current underwriting model (V2) was deployed in December 2025 and is the model that originates the portfolio today; earlier vintages were originated under the prior model.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A19:I19"/>
-    <mergeCell ref="A17:I17"/>
-    <mergeCell ref="A18:I18"/>
-    <mergeCell ref="A20:I20"/>
-    <mergeCell ref="A21:I21"/>
+    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A19:H19"/>
+    <mergeCell ref="A17:H17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2497,7 +2373,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Principal on accounts 90 or more days past due today, divided by originated principal on statements whose due date is at least 90 days old, for origination months January–September 2026 (in practice January–June, the vintages old enough to be measured). Shown for all accounts and excluding first-payment defaults; the window, the seasoning rule and the FPD definition are set out on the Loss Rate tab. Gross of recoveries; no balances have been written off to date (full provision at 180 DPD).</t>
+          <t>Principal on accounts 90 or more days past due today, divided by originated principal on statements whose due date is at least 90 days old, for origination months January–September 2026 (in practice January–June, the vintages old enough to be measured), excluding first-payment-default accounts from both numerator and denominator. The window, the seasoning rule and the FPD definition are set out on the Loss Rate tab, which also shows the FPD principal excluded. Gross of recoveries; no balances have been written off to date (full provision at 180 DPD).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Item 16: Jul/Aug/Sep/Q3 columns; interchange as rate × purchase turnover; tracker v29
</commit_message>
<xml_diff>
--- a/Prior Responses (outside data room)/Zed Portfolio Yield Analysis_20261027_DRAFT.xlsx
+++ b/Prior Responses (outside data room)/Zed Portfolio Yield Analysis_20261027_DRAFT.xlsx
@@ -108,12 +108,14 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -487,15 +489,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:J37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="60" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="58" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="66" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -508,7 +514,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gross and net yield on average receivables outstanding, annualized. September 2026 run-rate alongside January–September 2026. PHP; before operating, servicing and funding costs.</t>
+          <t>Gross and net yield on average receivables outstanding, annualized. July, August and September 2026 and the quarter together. PHP; before operating, servicing and funding costs.</t>
         </is>
       </c>
     </row>
@@ -517,25 +523,45 @@
       <c r="A4" s="3" t="inlineStr"/>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>September 2026</t>
+          <t>Jul 2026</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Annualized yield</t>
+          <t>Annualized</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Jan–Sep 2026</t>
+          <t>Aug 2026</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Annualized yield</t>
+          <t>Annualized</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Annualized</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Jul–Sep 2026</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Annualized</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -551,33 +577,47 @@
         <v>1</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" ht="48" customHeight="1">
+        <v>1</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
       <c r="A6" t="inlineStr">
         <is>
           <t>Average receivables outstanding</t>
         </is>
       </c>
       <c r="B6" s="5">
+        <f>'Monthly Detail'!H13</f>
+        <v/>
+      </c>
+      <c r="D6" s="5">
+        <f>'Monthly Detail'!I13</f>
+        <v/>
+      </c>
+      <c r="F6" s="5">
         <f>'Monthly Detail'!J13</f>
         <v/>
       </c>
-      <c r="D6" s="5">
+      <c r="H6" s="5">
         <f>'Monthly Detail'!K13</f>
         <v/>
       </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>Monthly average of daily receivables; Jan–Sep is the average of the nine monthly averages.</t>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>Monthly average of daily receivables; the quarter is the average of the three monthly averages.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>Revenue</t>
+          <t>Interest and fees — earned on balances</t>
         </is>
       </c>
       <c r="B7" s="8" t="n"/>
@@ -585,15 +625,19 @@
       <c r="D7" s="8" t="n"/>
       <c r="E7" s="8" t="n"/>
       <c r="F7" s="8" t="n"/>
-    </row>
-    <row r="8" ht="48" customHeight="1">
+      <c r="G7" s="8" t="n"/>
+      <c r="H7" s="8" t="n"/>
+      <c r="I7" s="8" t="n"/>
+      <c r="J7" s="8" t="n"/>
+    </row>
+    <row r="8" ht="34" customHeight="1">
       <c r="A8" t="inlineStr">
         <is>
           <t>Revolving interest</t>
         </is>
       </c>
       <c r="B8" s="5">
-        <f>'Monthly Detail'!J5</f>
+        <f>'Monthly Detail'!H5</f>
         <v/>
       </c>
       <c r="C8" s="9">
@@ -601,27 +645,43 @@
         <v/>
       </c>
       <c r="D8" s="5">
-        <f>'Monthly Detail'!K5</f>
+        <f>'Monthly Detail'!I5</f>
         <v/>
       </c>
       <c r="E8" s="9">
         <f>D8*12/D$5/D$6</f>
         <v/>
       </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>3% per month on revolving balances (BSP cap). Introduced with the June 2026 statement cycle, so the Jan–Sep figure covers four months of billing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="48" customHeight="1">
+      <c r="F8" s="5">
+        <f>'Monthly Detail'!J5</f>
+        <v/>
+      </c>
+      <c r="G8" s="9">
+        <f>F8*12/F$5/F$6</f>
+        <v/>
+      </c>
+      <c r="H8" s="5">
+        <f>'Monthly Detail'!K5</f>
+        <v/>
+      </c>
+      <c r="I8" s="9">
+        <f>H8*12/H$5/H$6</f>
+        <v/>
+      </c>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>3% per month on revolving balances (BSP cap). Introduced with the June 2026 statement cycle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
       <c r="A9" t="inlineStr">
         <is>
           <t>Installment interest</t>
         </is>
       </c>
       <c r="B9" s="5">
-        <f>'Monthly Detail'!J6</f>
+        <f>'Monthly Detail'!H6</f>
         <v/>
       </c>
       <c r="C9" s="9">
@@ -629,27 +689,43 @@
         <v/>
       </c>
       <c r="D9" s="5">
-        <f>'Monthly Detail'!K6</f>
+        <f>'Monthly Detail'!I6</f>
         <v/>
       </c>
       <c r="E9" s="9">
         <f>D9*12/D$5/D$6</f>
         <v/>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F9" s="5">
+        <f>'Monthly Detail'!J6</f>
+        <v/>
+      </c>
+      <c r="G9" s="9">
+        <f>F9*12/F$5/F$6</f>
+        <v/>
+      </c>
+      <c r="H9" s="5">
+        <f>'Monthly Detail'!K6</f>
+        <v/>
+      </c>
+      <c r="I9" s="9">
+        <f>H9*12/H$5/H$6</f>
+        <v/>
+      </c>
+      <c r="J9" s="6" t="inlineStr">
         <is>
           <t>1% per month on installment balances.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="48" customHeight="1">
+    <row r="10">
       <c r="A10" t="inlineStr">
         <is>
           <t>Installment upfront fees</t>
         </is>
       </c>
       <c r="B10" s="5">
-        <f>'Monthly Detail'!J7</f>
+        <f>'Monthly Detail'!H7</f>
         <v/>
       </c>
       <c r="C10" s="9">
@@ -657,14 +733,30 @@
         <v/>
       </c>
       <c r="D10" s="5">
-        <f>'Monthly Detail'!K7</f>
+        <f>'Monthly Detail'!I7</f>
         <v/>
       </c>
       <c r="E10" s="9">
         <f>D10*12/D$5/D$6</f>
         <v/>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F10" s="5">
+        <f>'Monthly Detail'!J7</f>
+        <v/>
+      </c>
+      <c r="G10" s="9">
+        <f>F10*12/F$5/F$6</f>
+        <v/>
+      </c>
+      <c r="H10" s="5">
+        <f>'Monthly Detail'!K7</f>
+        <v/>
+      </c>
+      <c r="I10" s="9">
+        <f>H10*12/H$5/H$6</f>
+        <v/>
+      </c>
+      <c r="J10" s="6" t="inlineStr">
         <is>
           <t>0.5% × term in months, billed at conversion.</t>
         </is>
@@ -677,7 +769,7 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>'Monthly Detail'!J8</f>
+        <f>'Monthly Detail'!H8</f>
         <v/>
       </c>
       <c r="C11" s="9">
@@ -685,13 +777,29 @@
         <v/>
       </c>
       <c r="D11" s="5">
-        <f>'Monthly Detail'!K8</f>
+        <f>'Monthly Detail'!I8</f>
         <v/>
       </c>
       <c r="E11" s="9">
         <f>D11*12/D$5/D$6</f>
         <v/>
       </c>
+      <c r="F11" s="5">
+        <f>'Monthly Detail'!J8</f>
+        <v/>
+      </c>
+      <c r="G11" s="9">
+        <f>F11*12/F$5/F$6</f>
+        <v/>
+      </c>
+      <c r="H11" s="5">
+        <f>'Monthly Detail'!K8</f>
+        <v/>
+      </c>
+      <c r="I11" s="9">
+        <f>H11*12/H$5/H$6</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -715,109 +823,173 @@
         <f>D12*12/D$5/D$6</f>
         <v/>
       </c>
-    </row>
-    <row r="13" ht="48" customHeight="1">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Interchange</t>
-        </is>
-      </c>
-      <c r="B13" s="5">
+      <c r="F12" s="11">
+        <f>SUM(F8:F11)</f>
+        <v/>
+      </c>
+      <c r="G12" s="12">
+        <f>F12*12/F$5/F$6</f>
+        <v/>
+      </c>
+      <c r="H12" s="11">
+        <f>SUM(H8:H11)</f>
+        <v/>
+      </c>
+      <c r="I12" s="12">
+        <f>H12*12/H$5/H$6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Interchange — earned on purchases, so a function of turnover</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="n"/>
+      <c r="C14" s="8" t="n"/>
+      <c r="D14" s="8" t="n"/>
+      <c r="E14" s="8" t="n"/>
+      <c r="F14" s="8" t="n"/>
+      <c r="G14" s="8" t="n"/>
+      <c r="H14" s="8" t="n"/>
+      <c r="I14" s="8" t="n"/>
+      <c r="J14" s="8" t="n"/>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Purchase volume settled</t>
+        </is>
+      </c>
+      <c r="B15" s="5">
+        <f>'Monthly Detail'!H16</f>
+        <v/>
+      </c>
+      <c r="D15" s="5">
+        <f>'Monthly Detail'!I16</f>
+        <v/>
+      </c>
+      <c r="F15" s="5">
+        <f>'Monthly Detail'!J16</f>
+        <v/>
+      </c>
+      <c r="H15" s="5">
+        <f>'Monthly Detail'!K16</f>
+        <v/>
+      </c>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>Cardholder purchases settled through Mastercard, net of returns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Purchase turnover (annualized purchase volume ÷ average receivables)</t>
+        </is>
+      </c>
+      <c r="C16" s="13">
+        <f>B15*12/B$5/B$6</f>
+        <v/>
+      </c>
+      <c r="E16" s="13">
+        <f>D15*12/D$5/D$6</f>
+        <v/>
+      </c>
+      <c r="G16" s="13">
+        <f>F15*12/F$5/F$6</f>
+        <v/>
+      </c>
+      <c r="I16" s="13">
+        <f>H15*12/H$5/H$6</f>
+        <v/>
+      </c>
+      <c r="J16" s="6" t="inlineStr">
+        <is>
+          <t>How many times a year the book is re-spent. Falls as more of the book revolves.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Interchange rate on purchase volume</t>
+        </is>
+      </c>
+      <c r="C17" s="14">
+        <f>B18/B15</f>
+        <v/>
+      </c>
+      <c r="E17" s="14">
+        <f>D18/D15</f>
+        <v/>
+      </c>
+      <c r="G17" s="14">
+        <f>F18/F15</f>
+        <v/>
+      </c>
+      <c r="I17" s="14">
+        <f>H18/H15</f>
+        <v/>
+      </c>
+      <c r="J17" s="6" t="inlineStr">
+        <is>
+          <t>Set by Mastercard by merchant category and domestic/foreign; gross of network and processing costs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="80" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Interchange income</t>
+        </is>
+      </c>
+      <c r="B18" s="11">
+        <f>'Monthly Detail'!H9</f>
+        <v/>
+      </c>
+      <c r="C18" s="12">
+        <f>C17*C16</f>
+        <v/>
+      </c>
+      <c r="D18" s="11">
+        <f>'Monthly Detail'!I9</f>
+        <v/>
+      </c>
+      <c r="E18" s="12">
+        <f>E17*E16</f>
+        <v/>
+      </c>
+      <c r="F18" s="11">
         <f>'Monthly Detail'!J9</f>
         <v/>
       </c>
-      <c r="C13" s="9">
-        <f>B13*12/B$5/B$6</f>
-        <v/>
-      </c>
-      <c r="D13" s="5">
+      <c r="G18" s="12">
+        <f>G17*G16</f>
+        <v/>
+      </c>
+      <c r="H18" s="11">
         <f>'Monthly Detail'!K9</f>
         <v/>
       </c>
-      <c r="E13" s="9">
-        <f>D13*12/D$5/D$6</f>
-        <v/>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>Earned on every purchase. Mastercard settles each purchase to the merchant net of interchange and the cardholder is billed the full purchase amount, so interchange is collected through cardholder payments.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="13" t="inlineStr">
-        <is>
-          <t>Total revenue</t>
-        </is>
-      </c>
-      <c r="B14" s="14">
-        <f>B12+B13</f>
-        <v/>
-      </c>
-      <c r="C14" s="15">
-        <f>B14*12/B$5/B$6</f>
-        <v/>
-      </c>
-      <c r="D14" s="14">
-        <f>D12+D13</f>
-        <v/>
-      </c>
-      <c r="E14" s="15">
-        <f>D14*12/D$5/D$6</f>
-        <v/>
-      </c>
-      <c r="F14" s="16" t="n"/>
-    </row>
-    <row r="15"/>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>Gross yield (annualized, on average receivables)</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="n"/>
-      <c r="C16" s="8" t="n"/>
-      <c r="D16" s="8" t="n"/>
-      <c r="E16" s="8" t="n"/>
-      <c r="F16" s="8" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Gross yield — interest and fees</t>
-        </is>
-      </c>
-      <c r="C17" s="9">
-        <f>C12</f>
-        <v/>
-      </c>
-      <c r="E17" s="9">
-        <f>E12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>Gross yield — all revenue, including interchange</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="n"/>
-      <c r="C18" s="12">
-        <f>C14</f>
-        <v/>
-      </c>
-      <c r="D18" s="10" t="n"/>
-      <c r="E18" s="12">
-        <f>E14</f>
-        <v/>
+      <c r="I18" s="12">
+        <f>I17*I16</f>
+        <v/>
+      </c>
+      <c r="J18" s="6" t="inlineStr">
+        <is>
+          <t>Yield on receivables = interchange rate × purchase turnover. Mastercard settles each purchase to the merchant net of interchange and the cardholder is billed the full amount, so interchange is collected through cardholder payments. It is earned once, when the receivable is created; a balance that then revolves earns interest, not further interchange.</t>
+        </is>
       </c>
     </row>
     <row r="19"/>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>Loss on receivables</t>
+          <t>Gross yield (annualized, on average receivables)</t>
         </is>
       </c>
       <c r="B20" s="8" t="n"/>
@@ -825,185 +997,357 @@
       <c r="D20" s="8" t="n"/>
       <c r="E20" s="8" t="n"/>
       <c r="F20" s="8" t="n"/>
+      <c r="G20" s="8" t="n"/>
+      <c r="H20" s="8" t="n"/>
+      <c r="I20" s="8" t="n"/>
+      <c r="J20" s="8" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>Gross yield — interest and fees</t>
+        </is>
+      </c>
+      <c r="C21" s="9">
+        <f>C12</f>
+        <v/>
+      </c>
+      <c r="E21" s="9">
+        <f>E12</f>
+        <v/>
+      </c>
+      <c r="G21" s="9">
+        <f>G12</f>
+        <v/>
+      </c>
+      <c r="I21" s="9">
+        <f>I12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>Gross yield — all revenue, including interchange</t>
+        </is>
+      </c>
+      <c r="B22" s="16">
+        <f>B12+B18</f>
+        <v/>
+      </c>
+      <c r="C22" s="17">
+        <f>C12+C18</f>
+        <v/>
+      </c>
+      <c r="D22" s="16">
+        <f>D12+D18</f>
+        <v/>
+      </c>
+      <c r="E22" s="17">
+        <f>E12+E18</f>
+        <v/>
+      </c>
+      <c r="F22" s="16">
+        <f>F12+F18</f>
+        <v/>
+      </c>
+      <c r="G22" s="17">
+        <f>G12+G18</f>
+        <v/>
+      </c>
+      <c r="H22" s="16">
+        <f>H12+H18</f>
+        <v/>
+      </c>
+      <c r="I22" s="17">
+        <f>I12+I18</f>
+        <v/>
+      </c>
+      <c r="J22" s="18" t="inlineStr">
+        <is>
+          <t>Amount column: total revenue for the period (ties to Monthly Detail).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23"/>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Loss on receivables — also a function of turnover</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="n"/>
+      <c r="C24" s="8" t="n"/>
+      <c r="D24" s="8" t="n"/>
+      <c r="E24" s="8" t="n"/>
+      <c r="F24" s="8" t="n"/>
+      <c r="G24" s="8" t="n"/>
+      <c r="H24" s="8" t="n"/>
+      <c r="I24" s="8" t="n"/>
+      <c r="J24" s="8" t="n"/>
+    </row>
+    <row r="25" ht="34" customHeight="1">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>Principal originated in period</t>
         </is>
       </c>
-      <c r="B21" s="5">
+      <c r="B25" s="5">
+        <f>'Monthly Detail'!H15</f>
+        <v/>
+      </c>
+      <c r="D25" s="5">
+        <f>'Monthly Detail'!I15</f>
+        <v/>
+      </c>
+      <c r="F25" s="5">
         <f>'Monthly Detail'!J15</f>
         <v/>
       </c>
-      <c r="D21" s="5">
+      <c r="H25" s="5">
         <f>'Monthly Detail'!K15</f>
         <v/>
       </c>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>Purchases billed to cardholders, net of refunds and chargebacks.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="48" customHeight="1">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Principal turnover (annualized originations ÷ average receivables)</t>
-        </is>
-      </c>
-      <c r="C22" s="17">
-        <f>B21*12/B5/B6</f>
-        <v/>
-      </c>
-      <c r="E22" s="17">
-        <f>D21*12/D5/D6</f>
-        <v/>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
-        <is>
-          <t>A card book turns over quickly: each peso of receivables is re-lent several times a year, so a loss rate on originations must be multiplied by turnover to compare it with a yield on balances.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="64" customHeight="1">
-      <c r="A23" t="inlineStr">
+      <c r="J25" s="6" t="inlineStr">
+        <is>
+          <t>Purchases billed to cardholders, net of refunds, chargebacks and cancelled-plan re-bookings; lower than purchase volume by definition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="34" customHeight="1">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Principal turnover (annualized originated principal ÷ average receivables)</t>
+        </is>
+      </c>
+      <c r="C26" s="13">
+        <f>B25*12/B$5/B$6</f>
+        <v/>
+      </c>
+      <c r="E26" s="13">
+        <f>D25*12/D$5/D$6</f>
+        <v/>
+      </c>
+      <c r="G26" s="13">
+        <f>F25*12/F$5/F$6</f>
+        <v/>
+      </c>
+      <c r="I26" s="13">
+        <f>H25*12/H$5/H$6</f>
+        <v/>
+      </c>
+      <c r="J26" s="6" t="inlineStr">
+        <is>
+          <t>Each peso of receivables is re-lent several times a year, so a loss rate on originations must be multiplied by turnover to compare it with a yield on balances.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="80" customHeight="1">
+      <c r="A27" t="inlineStr">
         <is>
           <t>Loss rate on originated principal — ≥90 DPD, excluding first-payment defaults</t>
         </is>
       </c>
-      <c r="C23" s="18">
+      <c r="C27" s="14">
         <f>loss_rate_xfpd</f>
         <v/>
       </c>
-      <c r="E23" s="18">
+      <c r="E27" s="14">
         <f>loss_rate_xfpd</f>
         <v/>
       </c>
-      <c r="F23" s="6" t="inlineStr">
-        <is>
-          <t>See the Loss Rate tab. Principal 90+ days past due ÷ originated principal on statements whose due date is ≥90 days old, vintages since January 2026, gross of recoveries; first-payment-default accounts (never made a payment; fraud/identity rather than credit) excluded from numerator and denominator. The same rate is applied to both periods.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24"/>
-    <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>Net yield (gross yield less loss on receivables)</t>
-        </is>
-      </c>
-      <c r="B25" s="8" t="n"/>
-      <c r="C25" s="8" t="n"/>
-      <c r="D25" s="8" t="n"/>
-      <c r="E25" s="8" t="n"/>
-      <c r="F25" s="8" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Loss on receivables (loss rate × turnover)</t>
-        </is>
-      </c>
-      <c r="C26" s="9">
-        <f>C23*C22</f>
-        <v/>
-      </c>
-      <c r="E26" s="9">
-        <f>E23*E22</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="10" t="inlineStr">
-        <is>
-          <t>Net yield — all revenue, including interchange</t>
-        </is>
-      </c>
-      <c r="B27" s="10" t="n"/>
-      <c r="C27" s="12">
-        <f>C18-C26</f>
-        <v/>
-      </c>
-      <c r="D27" s="10" t="n"/>
-      <c r="E27" s="12">
-        <f>E18-E26</f>
-        <v/>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
+      <c r="G27" s="14">
+        <f>loss_rate_xfpd</f>
+        <v/>
+      </c>
+      <c r="I27" s="14">
+        <f>loss_rate_xfpd</f>
+        <v/>
+      </c>
+      <c r="J27" s="6" t="inlineStr">
+        <is>
+          <t>See the Loss Rate tab. Principal 90+ days past due ÷ originated principal on statements whose due date is ≥90 days old, vintages since January 2026, gross of recoveries; first-payment-default accounts (never made a payment; fraud/identity rather than credit) excluded from numerator and denominator. The same rate is applied to every period.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>Loss on receivables (loss rate × principal turnover)</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="n"/>
+      <c r="C28" s="12">
+        <f>C27*C26</f>
+        <v/>
+      </c>
+      <c r="D28" s="10" t="n"/>
+      <c r="E28" s="12">
+        <f>E27*E26</f>
+        <v/>
+      </c>
+      <c r="F28" s="10" t="n"/>
+      <c r="G28" s="12">
+        <f>G27*G26</f>
+        <v/>
+      </c>
+      <c r="H28" s="10" t="n"/>
+      <c r="I28" s="12">
+        <f>I27*I26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29"/>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>Net yield</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="n"/>
+      <c r="C30" s="8" t="n"/>
+      <c r="D30" s="8" t="n"/>
+      <c r="E30" s="8" t="n"/>
+      <c r="F30" s="8" t="n"/>
+      <c r="G30" s="8" t="n"/>
+      <c r="H30" s="8" t="n"/>
+      <c r="I30" s="8" t="n"/>
+      <c r="J30" s="8" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>Net yield — all revenue less loss on receivables</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="n"/>
+      <c r="C31" s="12">
+        <f>C22-C28</f>
+        <v/>
+      </c>
+      <c r="D31" s="10" t="n"/>
+      <c r="E31" s="12">
+        <f>E22-E28</f>
+        <v/>
+      </c>
+      <c r="F31" s="10" t="n"/>
+      <c r="G31" s="12">
+        <f>G22-G28</f>
+        <v/>
+      </c>
+      <c r="H31" s="10" t="n"/>
+      <c r="I31" s="12">
+        <f>I22-I28</f>
+        <v/>
+      </c>
+      <c r="J31" s="6" t="inlineStr">
         <is>
           <t>Before operating, servicing and funding costs.</t>
         </is>
       </c>
     </row>
-    <row r="28"/>
-    <row r="29">
-      <c r="A29" s="7" t="inlineStr">
+    <row r="32"/>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
         <is>
           <t>Memo — USD equivalents</t>
         </is>
       </c>
-      <c r="B29" s="8" t="n"/>
-      <c r="C29" s="8" t="n"/>
-      <c r="D29" s="8" t="n"/>
-      <c r="E29" s="8" t="n"/>
-      <c r="F29" s="8" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="B33" s="8" t="n"/>
+      <c r="C33" s="8" t="n"/>
+      <c r="D33" s="8" t="n"/>
+      <c r="E33" s="8" t="n"/>
+      <c r="F33" s="8" t="n"/>
+      <c r="G33" s="8" t="n"/>
+      <c r="H33" s="8" t="n"/>
+      <c r="I33" s="8" t="n"/>
+      <c r="J33" s="8" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
         <is>
           <t>PHP per USD</t>
         </is>
       </c>
-      <c r="B30" s="19" t="n">
+      <c r="B34" s="19" t="n">
         <v>55.8</v>
       </c>
-      <c r="D30" s="19" t="n">
+      <c r="D34" s="19" t="n">
         <v>55.8</v>
       </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="F34" s="19" t="n">
+        <v>55.8</v>
+      </c>
+      <c r="H34" s="19" t="n">
+        <v>55.8</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
         <is>
           <t>Average receivables outstanding (USD)</t>
         </is>
       </c>
-      <c r="B31" s="5">
-        <f>B6/B30</f>
-        <v/>
-      </c>
-      <c r="D31" s="5">
-        <f>D6/D30</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="B35" s="5">
+        <f>B6/B34</f>
+        <v/>
+      </c>
+      <c r="D35" s="5">
+        <f>D6/D34</f>
+        <v/>
+      </c>
+      <c r="F35" s="5">
+        <f>F6/F34</f>
+        <v/>
+      </c>
+      <c r="H35" s="5">
+        <f>H6/H34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
         <is>
           <t>Total revenue (USD)</t>
         </is>
       </c>
-      <c r="B32" s="5">
-        <f>B14/B30</f>
-        <v/>
-      </c>
-      <c r="D32" s="5">
-        <f>D14/D30</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Principal originated (USD)</t>
-        </is>
-      </c>
-      <c r="B33" s="5">
-        <f>B21/B30</f>
-        <v/>
-      </c>
-      <c r="D33" s="5">
-        <f>D21/D30</f>
+      <c r="B36" s="5">
+        <f>B22/B34</f>
+        <v/>
+      </c>
+      <c r="D36" s="5">
+        <f>D22/D34</f>
+        <v/>
+      </c>
+      <c r="F36" s="5">
+        <f>F22/F34</f>
+        <v/>
+      </c>
+      <c r="H36" s="5">
+        <f>H22/H34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Purchase volume settled (USD)</t>
+        </is>
+      </c>
+      <c r="B37" s="5">
+        <f>B15/B34</f>
+        <v/>
+      </c>
+      <c r="D37" s="5">
+        <f>D15/D34</f>
+        <v/>
+      </c>
+      <c r="F37" s="5">
+        <f>F15/F34</f>
+        <v/>
+      </c>
+      <c r="H37" s="5">
+        <f>H15/H34</f>
         <v/>
       </c>
     </row>
@@ -1018,7 +1362,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K26"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -1102,7 +1446,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Jan–Sep 2026</t>
+          <t>Jul–Sep 2026</t>
         </is>
       </c>
     </row>
@@ -1140,7 +1484,7 @@
         <v>2229680.03</v>
       </c>
       <c r="K5" s="5">
-        <f>SUM(B5:J5)</f>
+        <f>SUM(H5:J5)</f>
         <v/>
       </c>
     </row>
@@ -1178,7 +1522,7 @@
         <v>486325.05</v>
       </c>
       <c r="K6" s="5">
-        <f>SUM(B6:J6)</f>
+        <f>SUM(H6:J6)</f>
         <v/>
       </c>
     </row>
@@ -1216,7 +1560,7 @@
         <v>439733.93</v>
       </c>
       <c r="K7" s="5">
-        <f>SUM(B7:J7)</f>
+        <f>SUM(H7:J7)</f>
         <v/>
       </c>
     </row>
@@ -1254,7 +1598,7 @@
         <v>126426.4</v>
       </c>
       <c r="K8" s="5">
-        <f>SUM(B8:J8)</f>
+        <f>SUM(H8:J8)</f>
         <v/>
       </c>
     </row>
@@ -1292,7 +1636,7 @@
         <v>2630889.798</v>
       </c>
       <c r="K9" s="5">
-        <f>SUM(B9:J9)</f>
+        <f>SUM(H9:J9)</f>
         <v/>
       </c>
     </row>
@@ -1395,7 +1739,7 @@
         <v>211159156.895</v>
       </c>
       <c r="K13" s="5">
-        <f>AVERAGE(B13:J13)</f>
+        <f>AVERAGE(H13:J13)</f>
         <v/>
       </c>
     </row>
@@ -1471,7 +1815,7 @@
         <v>160221212.53</v>
       </c>
       <c r="K15" s="5">
-        <f>SUM(B15:J15)</f>
+        <f>SUM(H15:J15)</f>
         <v/>
       </c>
     </row>
@@ -1509,7 +1853,7 @@
         <v>190860991.79</v>
       </c>
       <c r="K16" s="5">
-        <f>SUM(B16:J16)</f>
+        <f>SUM(H16:J16)</f>
         <v/>
       </c>
     </row>
@@ -1565,7 +1909,7 @@
         <v>1</v>
       </c>
       <c r="K19" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">
@@ -1712,46 +2056,46 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Principal turnover (annualized originations ÷ average receivables)</t>
-        </is>
-      </c>
-      <c r="B23" s="17">
+          <t>Principal turnover (annualized originated principal ÷ average receivables)</t>
+        </is>
+      </c>
+      <c r="B23" s="13">
         <f>B15*12/B19/B13</f>
         <v/>
       </c>
-      <c r="C23" s="17">
+      <c r="C23" s="13">
         <f>C15*12/C19/C13</f>
         <v/>
       </c>
-      <c r="D23" s="17">
+      <c r="D23" s="13">
         <f>D15*12/D19/D13</f>
         <v/>
       </c>
-      <c r="E23" s="17">
+      <c r="E23" s="13">
         <f>E15*12/E19/E13</f>
         <v/>
       </c>
-      <c r="F23" s="17">
+      <c r="F23" s="13">
         <f>F15*12/F19/F13</f>
         <v/>
       </c>
-      <c r="G23" s="17">
+      <c r="G23" s="13">
         <f>G15*12/G19/G13</f>
         <v/>
       </c>
-      <c r="H23" s="17">
+      <c r="H23" s="13">
         <f>H15*12/H19/H13</f>
         <v/>
       </c>
-      <c r="I23" s="17">
+      <c r="I23" s="13">
         <f>I15*12/I19/I13</f>
         <v/>
       </c>
-      <c r="J23" s="17">
+      <c r="J23" s="13">
         <f>J15*12/J19/J13</f>
         <v/>
       </c>
-      <c r="K23" s="17">
+      <c r="K23" s="13">
         <f>K15*12/K19/K13</f>
         <v/>
       </c>
@@ -1759,55 +2103,102 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Interchange rate on purchase volume (memo)</t>
-        </is>
-      </c>
-      <c r="B24" s="18">
+          <t>Purchase turnover (annualized purchase volume ÷ average receivables)</t>
+        </is>
+      </c>
+      <c r="B24" s="13">
+        <f>B16*12/B19/B13</f>
+        <v/>
+      </c>
+      <c r="C24" s="13">
+        <f>C16*12/C19/C13</f>
+        <v/>
+      </c>
+      <c r="D24" s="13">
+        <f>D16*12/D19/D13</f>
+        <v/>
+      </c>
+      <c r="E24" s="13">
+        <f>E16*12/E19/E13</f>
+        <v/>
+      </c>
+      <c r="F24" s="13">
+        <f>F16*12/F19/F13</f>
+        <v/>
+      </c>
+      <c r="G24" s="13">
+        <f>G16*12/G19/G13</f>
+        <v/>
+      </c>
+      <c r="H24" s="13">
+        <f>H16*12/H19/H13</f>
+        <v/>
+      </c>
+      <c r="I24" s="13">
+        <f>I16*12/I19/I13</f>
+        <v/>
+      </c>
+      <c r="J24" s="13">
+        <f>J16*12/J19/J13</f>
+        <v/>
+      </c>
+      <c r="K24" s="13">
+        <f>K16*12/K19/K13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Interchange rate on purchase volume</t>
+        </is>
+      </c>
+      <c r="B25" s="14">
         <f>B9/B16</f>
         <v/>
       </c>
-      <c r="C24" s="18">
+      <c r="C25" s="14">
         <f>C9/C16</f>
         <v/>
       </c>
-      <c r="D24" s="18">
+      <c r="D25" s="14">
         <f>D9/D16</f>
         <v/>
       </c>
-      <c r="E24" s="18">
+      <c r="E25" s="14">
         <f>E9/E16</f>
         <v/>
       </c>
-      <c r="F24" s="18">
+      <c r="F25" s="14">
         <f>F9/F16</f>
         <v/>
       </c>
-      <c r="G24" s="18">
+      <c r="G25" s="14">
         <f>G9/G16</f>
         <v/>
       </c>
-      <c r="H24" s="18">
+      <c r="H25" s="14">
         <f>H9/H16</f>
         <v/>
       </c>
-      <c r="I24" s="18">
+      <c r="I25" s="14">
         <f>I9/I16</f>
         <v/>
       </c>
-      <c r="J24" s="18">
+      <c r="J25" s="14">
         <f>J9/J16</f>
         <v/>
       </c>
-      <c r="K24" s="18">
+      <c r="K25" s="14">
         <f>K9/K16</f>
         <v/>
       </c>
     </row>
-    <row r="25"/>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Revolving interest was introduced with the June 2026 statement cycle; statements before then carried no revolving interest, so the Jan–Sep column understates the current run-rate of what is now the largest revenue line.</t>
+    <row r="26"/>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Installment plans scaled from March 2026 and revolving interest was introduced with the June 2026 statement cycle, so July–September 2026 is the first quarter with every revenue line in place. Earlier months are shown for completeness.</t>
         </is>
       </c>
     </row>
@@ -1916,7 +2307,7 @@
       <c r="G5" s="5" t="n">
         <v>1577286.85</v>
       </c>
-      <c r="H5" s="18">
+      <c r="H5" s="14">
         <f>IF(F5=0,"not yet seasoned",G5/F5)</f>
         <v/>
       </c>
@@ -1945,7 +2336,7 @@
       <c r="G6" s="5" t="n">
         <v>685527.14</v>
       </c>
-      <c r="H6" s="18">
+      <c r="H6" s="14">
         <f>IF(F6=0,"not yet seasoned",G6/F6)</f>
         <v/>
       </c>
@@ -1974,7 +2365,7 @@
       <c r="G7" s="5" t="n">
         <v>1404938.62</v>
       </c>
-      <c r="H7" s="18">
+      <c r="H7" s="14">
         <f>IF(F7=0,"not yet seasoned",G7/F7)</f>
         <v/>
       </c>
@@ -2003,7 +2394,7 @@
       <c r="G8" s="5" t="n">
         <v>1471002.56</v>
       </c>
-      <c r="H8" s="18">
+      <c r="H8" s="14">
         <f>IF(F8=0,"not yet seasoned",G8/F8)</f>
         <v/>
       </c>
@@ -2032,7 +2423,7 @@
       <c r="G9" s="5" t="n">
         <v>1061583</v>
       </c>
-      <c r="H9" s="18">
+      <c r="H9" s="14">
         <f>IF(F9=0,"not yet seasoned",G9/F9)</f>
         <v/>
       </c>
@@ -2061,7 +2452,7 @@
       <c r="G10" s="5" t="n">
         <v>459463.31</v>
       </c>
-      <c r="H10" s="18">
+      <c r="H10" s="14">
         <f>IF(F10=0,"not yet seasoned",G10/F10)</f>
         <v/>
       </c>
@@ -2090,7 +2481,7 @@
       <c r="G11" s="5" t="n">
         <v>8828.190000000001</v>
       </c>
-      <c r="H11" s="18">
+      <c r="H11" s="14">
         <f>IF(F11=0,"not yet seasoned",G11/F11)</f>
         <v/>
       </c>
@@ -2119,7 +2510,7 @@
       <c r="G12" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="18">
+      <c r="H12" s="14">
         <f>IF(F12=0,"not yet seasoned",G12/F12)</f>
         <v/>
       </c>
@@ -2148,38 +2539,38 @@
       <c r="G13" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="18">
+      <c r="H13" s="14">
         <f>IF(F13=0,"not yet seasoned",G13/F13)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>Since January 2026 (all vintages above)</t>
         </is>
       </c>
-      <c r="B14" s="14">
+      <c r="B14" s="16">
         <f>SUM(B5:B13)</f>
         <v/>
       </c>
-      <c r="C14" s="14">
+      <c r="C14" s="16">
         <f>SUM(C5:C13)</f>
         <v/>
       </c>
-      <c r="D14" s="14">
+      <c r="D14" s="16">
         <f>SUM(D5:D13)</f>
         <v/>
       </c>
-      <c r="E14" s="14">
+      <c r="E14" s="16">
         <f>SUM(E5:E13)</f>
         <v/>
       </c>
-      <c r="F14" s="14">
+      <c r="F14" s="16">
         <f>SUM(F5:F13)</f>
         <v/>
       </c>
-      <c r="G14" s="14">
+      <c r="G14" s="16">
         <f>SUM(G5:G13)</f>
         <v/>
       </c>
@@ -2242,7 +2633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2269,7 +2660,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="30" customHeight="1">
+    <row r="4" ht="75" customHeight="1">
       <c r="A4" s="22" t="inlineStr">
         <is>
           <t>Scope</t>
@@ -2277,7 +2668,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Zed's Philippine credit card receivables, all cardholders, January–September 2026. All figures in PHP unless marked USD (converted at 55.8 for reference only).</t>
+          <t>Zed's Philippine credit card receivables, all cardholders. Yield Summary covers July, August and September 2026 and the quarter together — the first quarter with every revenue line in place (installment plans scaled from March 2026; revolving interest introduced with the June 2026 cycle). Monthly Detail shows January–September 2026. All figures in PHP unless marked USD (converted at 55.8 for reference only).</t>
         </is>
       </c>
     </row>
@@ -2289,7 +2680,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Monthly average of receivables outstanding (principal, interest and fees billed to cardholders, plus installment principal not yet billed). The January–September figure is the simple average of the nine monthly averages, and yields for that period are revenue for the nine months × 12 ÷ 9 ÷ that average.</t>
+          <t>Monthly average of receivables outstanding (principal, interest and fees billed to cardholders, plus installment principal not yet billed). The July–September figure is the simple average of the three monthly averages, and yields for the quarter are revenue for the three months × 12 ÷ 3 ÷ that average.</t>
         </is>
       </c>
     </row>
@@ -2341,7 +2732,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="75" customHeight="1">
+    <row r="10" ht="90" customHeight="1">
       <c r="A10" s="22" t="inlineStr">
         <is>
           <t>Interchange</t>
@@ -2349,77 +2740,89 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Interchange received from Mastercard on cardholder purchases, gross (network and processing costs are not netted). Interchange is paid at settlement: the merchant receives the purchase amount less interchange, and the cardholder is billed the full purchase amount, so the interchange margin is collected as part of the cardholder's payment. The memo line on the Monthly Detail tab shows the same income as a percentage of purchase volume (1.38% in September 2026).</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="45" customHeight="1">
+          <t>Interchange received from Mastercard on cardholder purchases, gross (network and processing costs are not netted). Interchange is earned when a purchase settles, not on balances, so its yield on receivables is shown as interchange rate on purchase volume × purchase turnover (annualized purchase volume ÷ average receivables) — the same construction as the loss line. Mastercard settles the merchant net of interchange and the cardholder is billed the full purchase amount, so the interchange margin is collected as part of the cardholder's payment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="60" customHeight="1">
       <c r="A11" s="22" t="inlineStr">
         <is>
+          <t>Purchase volume and turnover</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Purchase volume is cardholder spend settled through Mastercard, net of returns (the interchange base). Principal originated is purchases billed to cardholders net of refunds, chargebacks and cancelled installment-plan re-bookings (the loss base); it is lower than purchase volume by definition. Each is annualized and divided by average receivables to give its turnover.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="22" t="inlineStr">
+        <is>
           <t>Principal originated</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Purchases and other charges billed to cardholders in the month, net of refunds, chargebacks and cancelled installment plan re-bookings. Source: Zed's statement data, the same data underlying the statement tape in the data room.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="90" customHeight="1">
-      <c r="A12" s="22" t="inlineStr">
+    <row r="13" ht="90" customHeight="1">
+      <c r="A13" s="22" t="inlineStr">
         <is>
           <t>Loss rate</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Principal on accounts 90 or more days past due today, divided by originated principal on statements whose due date is at least 90 days old, for origination months January–September 2026 (in practice January–June, the vintages old enough to be measured), excluding first-payment-default accounts from both numerator and denominator. The window, the seasoning rule and the FPD definition are set out on the Loss Rate tab, which also shows the FPD principal excluded. Gross of recoveries; no balances have been written off to date (full provision at 180 DPD).</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="45" customHeight="1">
-      <c r="A13" s="22" t="inlineStr">
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="22" t="inlineStr">
         <is>
           <t>Loss on receivables</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Loss rate on originated principal × principal turnover (annualized originations ÷ average receivables). Expresses a loss on amounts lent as an annual charge against the receivables balance, on the same basis as the yields.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="22" t="inlineStr">
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="22" t="inlineStr">
         <is>
           <t>Net yield</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Gross yield less loss on receivables. Before operating costs, servicing, processing and network costs, funding costs, taxes and FX.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="60" customHeight="1">
-      <c r="A15" s="22" t="inlineStr">
+    <row r="16" ht="60" customHeight="1">
+      <c r="A16" s="22" t="inlineStr">
         <is>
           <t>Sources</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Zed management reporting built from the i2c transaction and settlement extracts (revenue, receivables, purchase volume; as of 26 October 2026) and Zed's statement and delinquency data (originations, delinquency by origination month; as of 27 October 2026). September 2026 is the latest complete month.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="22" t="inlineStr">
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="22" t="inlineStr">
         <is>
           <t>Prepared</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Zed Financial, October 2026. Prepared for Accial Capital in connection with its evaluation of a receivables facility.</t>
         </is>

</xml_diff>

<commit_message>
Item 16: calendar-month principal flow (purchase volume + pay-a-friend) as loss base; pay-a-friend CSV filed; tracker v30
</commit_message>
<xml_diff>
--- a/Prior Responses (outside data room)/Zed Portfolio Yield Analysis_20261027_DRAFT.xlsx
+++ b/Prior Responses (outside data room)/Zed Portfolio Yield Analysis_20261027_DRAFT.xlsx
@@ -1089,35 +1089,35 @@
     <row r="25" ht="34" customHeight="1">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Principal originated in period</t>
+          <t>Principal flow in period (purchase volume + pay-a-friend transfers)</t>
         </is>
       </c>
       <c r="B25" s="5">
-        <f>'Monthly Detail'!H15</f>
+        <f>'Monthly Detail'!H18</f>
         <v/>
       </c>
       <c r="D25" s="5">
-        <f>'Monthly Detail'!I15</f>
+        <f>'Monthly Detail'!I18</f>
         <v/>
       </c>
       <c r="F25" s="5">
-        <f>'Monthly Detail'!J15</f>
+        <f>'Monthly Detail'!J18</f>
         <v/>
       </c>
       <c r="H25" s="5">
-        <f>'Monthly Detail'!K15</f>
+        <f>'Monthly Detail'!K18</f>
         <v/>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
-          <t>Purchases billed to cardholders, net of refunds, chargebacks and cancelled-plan re-bookings; lower than purchase volume by definition.</t>
+          <t>Everything that became a receivable in the month: Mastercard purchases net of returns plus pay-a-friend transfers (which earn no interchange). Calendar-month, same basis as average receivables.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="34" customHeight="1">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Principal turnover (annualized originated principal ÷ average receivables)</t>
+          <t>Principal turnover (annualized principal flow ÷ average receivables)</t>
         </is>
       </c>
       <c r="C26" s="13">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>Each peso of receivables is re-lent several times a year, so a loss rate on originations must be multiplied by turnover to compare it with a yield on balances.</t>
+          <t>Each peso of receivables is re-lent several times a year, so a loss rate on originations must be multiplied by turnover to compare it with a yield on balances. Differs from purchase turnover only by pay-a-friend.</t>
         </is>
       </c>
     </row>
@@ -1331,23 +1331,23 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Purchase volume settled (USD)</t>
+          <t>Principal flow (USD)</t>
         </is>
       </c>
       <c r="B37" s="5">
-        <f>B15/B34</f>
+        <f>B25/B34</f>
         <v/>
       </c>
       <c r="D37" s="5">
-        <f>D15/D34</f>
+        <f>D25/D34</f>
         <v/>
       </c>
       <c r="F37" s="5">
-        <f>F15/F34</f>
+        <f>F25/F34</f>
         <v/>
       </c>
       <c r="H37" s="5">
-        <f>H15/H34</f>
+        <f>H25/H34</f>
         <v/>
       </c>
     </row>
@@ -1362,7 +1362,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -1784,7 +1784,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Principal originated (purchases billed, net of refunds and chargebacks)</t>
+          <t>Principal originated, statement-month basis (base on which the loss rate is measured)</t>
         </is>
       </c>
       <c r="B15" s="5" t="n">
@@ -1857,346 +1857,431 @@
         <v/>
       </c>
     </row>
-    <row r="17"/>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Pay-a-friend transfers (cardholder-to-cardholder, charged to the card; no interchange)</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>1060000</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>980000</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>1900000</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>1190000</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>2250000</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>2040000</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>2730000</v>
+      </c>
+      <c r="I17" s="5" t="n">
+        <v>2970000</v>
+      </c>
+      <c r="J17" s="5" t="n">
+        <v>2650000</v>
+      </c>
+      <c r="K17" s="5">
+        <f>SUM(H17:J17)</f>
+        <v/>
+      </c>
+    </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Principal flow (purchase volume + pay-a-friend) — calendar-month loss base</t>
+        </is>
+      </c>
+      <c r="B18" s="5">
+        <f>B16+B17</f>
+        <v/>
+      </c>
+      <c r="C18" s="5">
+        <f>C16+C17</f>
+        <v/>
+      </c>
+      <c r="D18" s="5">
+        <f>D16+D17</f>
+        <v/>
+      </c>
+      <c r="E18" s="5">
+        <f>E16+E17</f>
+        <v/>
+      </c>
+      <c r="F18" s="5">
+        <f>F16+F17</f>
+        <v/>
+      </c>
+      <c r="G18" s="5">
+        <f>G16+G17</f>
+        <v/>
+      </c>
+      <c r="H18" s="5">
+        <f>H16+H17</f>
+        <v/>
+      </c>
+      <c r="I18" s="5">
+        <f>I16+I17</f>
+        <v/>
+      </c>
+      <c r="J18" s="5">
+        <f>J16+J17</f>
+        <v/>
+      </c>
+      <c r="K18" s="5">
+        <f>K16+K17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>Annualized yields on average receivables</t>
         </is>
       </c>
-      <c r="B18" s="8" t="n"/>
-      <c r="C18" s="8" t="n"/>
-      <c r="D18" s="8" t="n"/>
-      <c r="E18" s="8" t="n"/>
-      <c r="F18" s="8" t="n"/>
-      <c r="G18" s="8" t="n"/>
-      <c r="H18" s="8" t="n"/>
-      <c r="I18" s="8" t="n"/>
-      <c r="J18" s="8" t="n"/>
-      <c r="K18" s="8" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Months in period</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C19" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" t="n">
-        <v>1</v>
-      </c>
-      <c r="G19" t="n">
-        <v>1</v>
-      </c>
-      <c r="H19" t="n">
-        <v>1</v>
-      </c>
-      <c r="I19" t="n">
-        <v>1</v>
-      </c>
-      <c r="J19" t="n">
-        <v>1</v>
-      </c>
-      <c r="K19" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Interest and fees (revolving + installment + late)</t>
-        </is>
-      </c>
-      <c r="B20" s="9">
-        <f>SUM(B5:B8)*12/B19/B13</f>
-        <v/>
-      </c>
-      <c r="C20" s="9">
-        <f>SUM(C5:C8)*12/C19/C13</f>
-        <v/>
-      </c>
-      <c r="D20" s="9">
-        <f>SUM(D5:D8)*12/D19/D13</f>
-        <v/>
-      </c>
-      <c r="E20" s="9">
-        <f>SUM(E5:E8)*12/E19/E13</f>
-        <v/>
-      </c>
-      <c r="F20" s="9">
-        <f>SUM(F5:F8)*12/F19/F13</f>
-        <v/>
-      </c>
-      <c r="G20" s="9">
-        <f>SUM(G5:G8)*12/G19/G13</f>
-        <v/>
-      </c>
-      <c r="H20" s="9">
-        <f>SUM(H5:H8)*12/H19/H13</f>
-        <v/>
-      </c>
-      <c r="I20" s="9">
-        <f>SUM(I5:I8)*12/I19/I13</f>
-        <v/>
-      </c>
-      <c r="J20" s="9">
-        <f>SUM(J5:J8)*12/J19/J13</f>
-        <v/>
-      </c>
-      <c r="K20" s="9">
-        <f>SUM(K5:K8)*12/K19/K13</f>
-        <v/>
-      </c>
+      <c r="B20" s="8" t="n"/>
+      <c r="C20" s="8" t="n"/>
+      <c r="D20" s="8" t="n"/>
+      <c r="E20" s="8" t="n"/>
+      <c r="F20" s="8" t="n"/>
+      <c r="G20" s="8" t="n"/>
+      <c r="H20" s="8" t="n"/>
+      <c r="I20" s="8" t="n"/>
+      <c r="J20" s="8" t="n"/>
+      <c r="K20" s="8" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Interchange</t>
-        </is>
-      </c>
-      <c r="B21" s="9">
-        <f>B9*12/B19/B13</f>
-        <v/>
-      </c>
-      <c r="C21" s="9">
-        <f>C9*12/C19/C13</f>
-        <v/>
-      </c>
-      <c r="D21" s="9">
-        <f>D9*12/D19/D13</f>
-        <v/>
-      </c>
-      <c r="E21" s="9">
-        <f>E9*12/E19/E13</f>
-        <v/>
-      </c>
-      <c r="F21" s="9">
-        <f>F9*12/F19/F13</f>
-        <v/>
-      </c>
-      <c r="G21" s="9">
-        <f>G9*12/G19/G13</f>
-        <v/>
-      </c>
-      <c r="H21" s="9">
-        <f>H9*12/H19/H13</f>
-        <v/>
-      </c>
-      <c r="I21" s="9">
-        <f>I9*12/I19/I13</f>
-        <v/>
-      </c>
-      <c r="J21" s="9">
-        <f>J9*12/J19/J13</f>
-        <v/>
-      </c>
-      <c r="K21" s="9">
-        <f>K9*12/K19/K13</f>
-        <v/>
+          <t>Months in period</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" t="n">
+        <v>1</v>
+      </c>
+      <c r="J21" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="inlineStr">
-        <is>
-          <t>Gross yield — all revenue</t>
-        </is>
-      </c>
-      <c r="B22" s="12">
-        <f>B10*12/B19/B13</f>
-        <v/>
-      </c>
-      <c r="C22" s="12">
-        <f>C10*12/C19/C13</f>
-        <v/>
-      </c>
-      <c r="D22" s="12">
-        <f>D10*12/D19/D13</f>
-        <v/>
-      </c>
-      <c r="E22" s="12">
-        <f>E10*12/E19/E13</f>
-        <v/>
-      </c>
-      <c r="F22" s="12">
-        <f>F10*12/F19/F13</f>
-        <v/>
-      </c>
-      <c r="G22" s="12">
-        <f>G10*12/G19/G13</f>
-        <v/>
-      </c>
-      <c r="H22" s="12">
-        <f>H10*12/H19/H13</f>
-        <v/>
-      </c>
-      <c r="I22" s="12">
-        <f>I10*12/I19/I13</f>
-        <v/>
-      </c>
-      <c r="J22" s="12">
-        <f>J10*12/J19/J13</f>
-        <v/>
-      </c>
-      <c r="K22" s="12">
-        <f>K10*12/K19/K13</f>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Interest and fees (revolving + installment + late)</t>
+        </is>
+      </c>
+      <c r="B22" s="9">
+        <f>SUM(B5:B8)*12/B21/B13</f>
+        <v/>
+      </c>
+      <c r="C22" s="9">
+        <f>SUM(C5:C8)*12/C21/C13</f>
+        <v/>
+      </c>
+      <c r="D22" s="9">
+        <f>SUM(D5:D8)*12/D21/D13</f>
+        <v/>
+      </c>
+      <c r="E22" s="9">
+        <f>SUM(E5:E8)*12/E21/E13</f>
+        <v/>
+      </c>
+      <c r="F22" s="9">
+        <f>SUM(F5:F8)*12/F21/F13</f>
+        <v/>
+      </c>
+      <c r="G22" s="9">
+        <f>SUM(G5:G8)*12/G21/G13</f>
+        <v/>
+      </c>
+      <c r="H22" s="9">
+        <f>SUM(H5:H8)*12/H21/H13</f>
+        <v/>
+      </c>
+      <c r="I22" s="9">
+        <f>SUM(I5:I8)*12/I21/I13</f>
+        <v/>
+      </c>
+      <c r="J22" s="9">
+        <f>SUM(J5:J8)*12/J21/J13</f>
+        <v/>
+      </c>
+      <c r="K22" s="9">
+        <f>SUM(K5:K8)*12/K21/K13</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Principal turnover (annualized originated principal ÷ average receivables)</t>
-        </is>
-      </c>
-      <c r="B23" s="13">
-        <f>B15*12/B19/B13</f>
-        <v/>
-      </c>
-      <c r="C23" s="13">
-        <f>C15*12/C19/C13</f>
-        <v/>
-      </c>
-      <c r="D23" s="13">
-        <f>D15*12/D19/D13</f>
-        <v/>
-      </c>
-      <c r="E23" s="13">
-        <f>E15*12/E19/E13</f>
-        <v/>
-      </c>
-      <c r="F23" s="13">
-        <f>F15*12/F19/F13</f>
-        <v/>
-      </c>
-      <c r="G23" s="13">
-        <f>G15*12/G19/G13</f>
-        <v/>
-      </c>
-      <c r="H23" s="13">
-        <f>H15*12/H19/H13</f>
-        <v/>
-      </c>
-      <c r="I23" s="13">
-        <f>I15*12/I19/I13</f>
-        <v/>
-      </c>
-      <c r="J23" s="13">
-        <f>J15*12/J19/J13</f>
-        <v/>
-      </c>
-      <c r="K23" s="13">
-        <f>K15*12/K19/K13</f>
+          <t>Interchange</t>
+        </is>
+      </c>
+      <c r="B23" s="9">
+        <f>B9*12/B21/B13</f>
+        <v/>
+      </c>
+      <c r="C23" s="9">
+        <f>C9*12/C21/C13</f>
+        <v/>
+      </c>
+      <c r="D23" s="9">
+        <f>D9*12/D21/D13</f>
+        <v/>
+      </c>
+      <c r="E23" s="9">
+        <f>E9*12/E21/E13</f>
+        <v/>
+      </c>
+      <c r="F23" s="9">
+        <f>F9*12/F21/F13</f>
+        <v/>
+      </c>
+      <c r="G23" s="9">
+        <f>G9*12/G21/G13</f>
+        <v/>
+      </c>
+      <c r="H23" s="9">
+        <f>H9*12/H21/H13</f>
+        <v/>
+      </c>
+      <c r="I23" s="9">
+        <f>I9*12/I21/I13</f>
+        <v/>
+      </c>
+      <c r="J23" s="9">
+        <f>J9*12/J21/J13</f>
+        <v/>
+      </c>
+      <c r="K23" s="9">
+        <f>K9*12/K21/K13</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Purchase turnover (annualized purchase volume ÷ average receivables)</t>
-        </is>
-      </c>
-      <c r="B24" s="13">
-        <f>B16*12/B19/B13</f>
-        <v/>
-      </c>
-      <c r="C24" s="13">
-        <f>C16*12/C19/C13</f>
-        <v/>
-      </c>
-      <c r="D24" s="13">
-        <f>D16*12/D19/D13</f>
-        <v/>
-      </c>
-      <c r="E24" s="13">
-        <f>E16*12/E19/E13</f>
-        <v/>
-      </c>
-      <c r="F24" s="13">
-        <f>F16*12/F19/F13</f>
-        <v/>
-      </c>
-      <c r="G24" s="13">
-        <f>G16*12/G19/G13</f>
-        <v/>
-      </c>
-      <c r="H24" s="13">
-        <f>H16*12/H19/H13</f>
-        <v/>
-      </c>
-      <c r="I24" s="13">
-        <f>I16*12/I19/I13</f>
-        <v/>
-      </c>
-      <c r="J24" s="13">
-        <f>J16*12/J19/J13</f>
-        <v/>
-      </c>
-      <c r="K24" s="13">
-        <f>K16*12/K19/K13</f>
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>Gross yield — all revenue</t>
+        </is>
+      </c>
+      <c r="B24" s="12">
+        <f>B10*12/B21/B13</f>
+        <v/>
+      </c>
+      <c r="C24" s="12">
+        <f>C10*12/C21/C13</f>
+        <v/>
+      </c>
+      <c r="D24" s="12">
+        <f>D10*12/D21/D13</f>
+        <v/>
+      </c>
+      <c r="E24" s="12">
+        <f>E10*12/E21/E13</f>
+        <v/>
+      </c>
+      <c r="F24" s="12">
+        <f>F10*12/F21/F13</f>
+        <v/>
+      </c>
+      <c r="G24" s="12">
+        <f>G10*12/G21/G13</f>
+        <v/>
+      </c>
+      <c r="H24" s="12">
+        <f>H10*12/H21/H13</f>
+        <v/>
+      </c>
+      <c r="I24" s="12">
+        <f>I10*12/I21/I13</f>
+        <v/>
+      </c>
+      <c r="J24" s="12">
+        <f>J10*12/J21/J13</f>
+        <v/>
+      </c>
+      <c r="K24" s="12">
+        <f>K10*12/K21/K13</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>Principal turnover (annualized principal flow ÷ average receivables)</t>
+        </is>
+      </c>
+      <c r="B25" s="13">
+        <f>B18*12/B21/B13</f>
+        <v/>
+      </c>
+      <c r="C25" s="13">
+        <f>C18*12/C21/C13</f>
+        <v/>
+      </c>
+      <c r="D25" s="13">
+        <f>D18*12/D21/D13</f>
+        <v/>
+      </c>
+      <c r="E25" s="13">
+        <f>E18*12/E21/E13</f>
+        <v/>
+      </c>
+      <c r="F25" s="13">
+        <f>F18*12/F21/F13</f>
+        <v/>
+      </c>
+      <c r="G25" s="13">
+        <f>G18*12/G21/G13</f>
+        <v/>
+      </c>
+      <c r="H25" s="13">
+        <f>H18*12/H21/H13</f>
+        <v/>
+      </c>
+      <c r="I25" s="13">
+        <f>I18*12/I21/I13</f>
+        <v/>
+      </c>
+      <c r="J25" s="13">
+        <f>J18*12/J21/J13</f>
+        <v/>
+      </c>
+      <c r="K25" s="13">
+        <f>K18*12/K21/K13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Purchase turnover (annualized purchase volume ÷ average receivables)</t>
+        </is>
+      </c>
+      <c r="B26" s="13">
+        <f>B16*12/B21/B13</f>
+        <v/>
+      </c>
+      <c r="C26" s="13">
+        <f>C16*12/C21/C13</f>
+        <v/>
+      </c>
+      <c r="D26" s="13">
+        <f>D16*12/D21/D13</f>
+        <v/>
+      </c>
+      <c r="E26" s="13">
+        <f>E16*12/E21/E13</f>
+        <v/>
+      </c>
+      <c r="F26" s="13">
+        <f>F16*12/F21/F13</f>
+        <v/>
+      </c>
+      <c r="G26" s="13">
+        <f>G16*12/G21/G13</f>
+        <v/>
+      </c>
+      <c r="H26" s="13">
+        <f>H16*12/H21/H13</f>
+        <v/>
+      </c>
+      <c r="I26" s="13">
+        <f>I16*12/I21/I13</f>
+        <v/>
+      </c>
+      <c r="J26" s="13">
+        <f>J16*12/J21/J13</f>
+        <v/>
+      </c>
+      <c r="K26" s="13">
+        <f>K16*12/K21/K13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>Interchange rate on purchase volume</t>
         </is>
       </c>
-      <c r="B25" s="14">
+      <c r="B27" s="14">
         <f>B9/B16</f>
         <v/>
       </c>
-      <c r="C25" s="14">
+      <c r="C27" s="14">
         <f>C9/C16</f>
         <v/>
       </c>
-      <c r="D25" s="14">
+      <c r="D27" s="14">
         <f>D9/D16</f>
         <v/>
       </c>
-      <c r="E25" s="14">
+      <c r="E27" s="14">
         <f>E9/E16</f>
         <v/>
       </c>
-      <c r="F25" s="14">
+      <c r="F27" s="14">
         <f>F9/F16</f>
         <v/>
       </c>
-      <c r="G25" s="14">
+      <c r="G27" s="14">
         <f>G9/G16</f>
         <v/>
       </c>
-      <c r="H25" s="14">
+      <c r="H27" s="14">
         <f>H9/H16</f>
         <v/>
       </c>
-      <c r="I25" s="14">
+      <c r="I27" s="14">
         <f>I9/I16</f>
         <v/>
       </c>
-      <c r="J25" s="14">
+      <c r="J27" s="14">
         <f>J9/J16</f>
         <v/>
       </c>
-      <c r="K25" s="14">
+      <c r="K27" s="14">
         <f>K9/K16</f>
         <v/>
       </c>
     </row>
-    <row r="26"/>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+    <row r="28"/>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>Installment plans scaled from March 2026 and revolving interest was introduced with the June 2026 statement cycle, so July–September 2026 is the first quarter with every revenue line in place. Earlier months are shown for completeness.</t>
         </is>
@@ -2633,7 +2718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2744,85 +2829,97 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="60" customHeight="1">
+    <row r="11" ht="45" customHeight="1">
       <c r="A11" s="22" t="inlineStr">
         <is>
-          <t>Purchase volume and turnover</t>
+          <t>Turnover</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Purchase volume is cardholder spend settled through Mastercard, net of returns (the interchange base). Principal originated is purchases billed to cardholders net of refunds, chargebacks and cancelled installment-plan re-bookings (the loss base); it is lower than purchase volume by definition. Each is annualized and divided by average receivables to give its turnover.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="45" customHeight="1">
+          <t>Annualized flow ÷ average receivables. Purchase turnover uses Mastercard purchase volume (the interchange base); principal turnover uses principal flow (the loss base). They differ only by pay-a-friend transfers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="60" customHeight="1">
       <c r="A12" s="22" t="inlineStr">
         <is>
-          <t>Principal originated</t>
+          <t>Principal flow</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Purchases and other charges billed to cardholders in the month, net of refunds, chargebacks and cancelled installment plan re-bookings. Source: Zed's statement data, the same data underlying the statement tape in the data room.</t>
+          <t>Calendar-month flow of new receivables: Mastercard purchase volume net of returns plus pay-a-friend transfers (cardholder-to-cardholder transfers charged to the card, which earn no interchange). This is the loss base in the Yield Summary and is on the same calendar basis as average receivables.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="90" customHeight="1">
       <c r="A13" s="22" t="inlineStr">
         <is>
+          <t>Principal originated (Loss Rate tab)</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>The same quantity measured by statement month: charges on statements closing in the month (cycles close on the 14th and the last day), net of refunds, chargebacks and cancelled installment-plan re-bookings. The loss rate is measured on this basis because delinquency is tracked by statement; a statement month covers roughly the second half of the prior calendar month and the first half of the current one, so individual months differ from the calendar flow by timing while the two agree over longer windows (Jan–Sep 2026: ₱1,025M vs ₱1,035M).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="90" customHeight="1">
+      <c r="A14" s="22" t="inlineStr">
+        <is>
           <t>Loss rate</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Principal on accounts 90 or more days past due today, divided by originated principal on statements whose due date is at least 90 days old, for origination months January–September 2026 (in practice January–June, the vintages old enough to be measured), excluding first-payment-default accounts from both numerator and denominator. The window, the seasoning rule and the FPD definition are set out on the Loss Rate tab, which also shows the FPD principal excluded. Gross of recoveries; no balances have been written off to date (full provision at 180 DPD).</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="45" customHeight="1">
-      <c r="A14" s="22" t="inlineStr">
+    <row r="15" ht="45" customHeight="1">
+      <c r="A15" s="22" t="inlineStr">
         <is>
           <t>Loss on receivables</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Loss rate on originated principal × principal turnover (annualized originations ÷ average receivables). Expresses a loss on amounts lent as an annual charge against the receivables balance, on the same basis as the yields.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="22" t="inlineStr">
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="22" t="inlineStr">
         <is>
           <t>Net yield</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Gross yield less loss on receivables. Before operating costs, servicing, processing and network costs, funding costs, taxes and FX.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="60" customHeight="1">
-      <c r="A16" s="22" t="inlineStr">
+    <row r="17" ht="60" customHeight="1">
+      <c r="A17" s="22" t="inlineStr">
         <is>
           <t>Sources</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>Zed management reporting built from the i2c transaction and settlement extracts (revenue, receivables, purchase volume; as of 26 October 2026) and Zed's statement and delinquency data (originations, delinquency by origination month; as of 27 October 2026). September 2026 is the latest complete month.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="22" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Zed management reporting built from the i2c transaction and settlement extracts (revenue, receivables, purchase volume; as of 26 October 2026), the processor transaction feed (pay-a-friend transfers) and Zed's statement and delinquency data (originations, delinquency by origination month; as of 27 October 2026). September 2026 is the latest complete month.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="22" t="inlineStr">
         <is>
           <t>Prepared</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Zed Financial, October 2026. Prepared for Accial Capital in connection with its evaluation of a receivables facility.</t>
         </is>

</xml_diff>

<commit_message>
Item 16: loss-emergence table on the Loss Rate tab; factual FPD-controls note from the handoff; ring Q&A only; tracker v31
</commit_message>
<xml_diff>
--- a/Prior Responses (outside data room)/Zed Portfolio Yield Analysis_20261027_DRAFT.xlsx
+++ b/Prior Responses (outside data room)/Zed Portfolio Yield Analysis_20261027_DRAFT.xlsx
@@ -90,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -121,6 +121,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
@@ -2298,11 +2302,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
@@ -2689,7 +2693,7 @@
     <row r="19" ht="48" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>• First-payment defaults (FPD). An account whose first-ever statement was the one missed, i.e. a cardholder who never made a payment. These are fraud or identity cases rather than credit losses and are excluded from the loss rate; the principal excluded is shown in column E so the adjustment is visible. Receivables of this kind would ordinarily fall outside facility eligibility criteria. Zed now manages first-payment default through dedicated onboarding and fraud controls, separately from credit underwriting.</t>
+          <t>• First-payment defaults (FPD). An account whose first-ever statement was the one missed, i.e. a cardholder who never made a payment. These are fraud or identity cases rather than credit losses and are excluded from the loss rate; the principal excluded is shown in column E so the adjustment is visible. Receivables of this kind would ordinarily fall outside facility eligibility criteria. First-payment default is managed separately from credit underwriting: duplicate-applicant checks (exact name and date of birth, ID number) have been in place since 1 October 2026, and from the 24 October 2026 decisioning run every application is screened for bank account numbers shared with another applicant, repeated selfie or ID images, invite-name mismatches and past-due bureau tradelines, with business-owner limits set on half of declared income pending documents.</t>
         </is>
       </c>
     </row>
@@ -2700,12 +2704,291 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Loss emergence — when a vintage's loss arrives (ex-FPD, same measure as the table above)</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="n"/>
+      <c r="C22" s="8" t="n"/>
+      <c r="D22" s="8" t="n"/>
+      <c r="E22" s="8" t="n"/>
+      <c r="F22" s="8" t="n"/>
+      <c r="G22" s="8" t="n"/>
+      <c r="H22" s="8" t="n"/>
+    </row>
+    <row r="23" ht="32" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Origination month</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>By month 3 on book</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>By month 4</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>By month 5</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>By month 6</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>By month 8</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Today</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Months on book today</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Jan 2026</t>
+        </is>
+      </c>
+      <c r="B24" s="22" t="n">
+        <v>0.00675</v>
+      </c>
+      <c r="C24" s="22" t="n">
+        <v>0.02263</v>
+      </c>
+      <c r="D24" s="22" t="n">
+        <v>0.02263</v>
+      </c>
+      <c r="E24" s="22" t="n">
+        <v>0.02263</v>
+      </c>
+      <c r="F24" s="22" t="n">
+        <v>0.02263</v>
+      </c>
+      <c r="G24" s="23" t="n">
+        <v>0.02263</v>
+      </c>
+      <c r="H24" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Feb 2026</t>
+        </is>
+      </c>
+      <c r="B25" s="22" t="n">
+        <v>0.00851</v>
+      </c>
+      <c r="C25" s="22" t="n">
+        <v>0.01028</v>
+      </c>
+      <c r="D25" s="22" t="n">
+        <v>0.01118</v>
+      </c>
+      <c r="E25" s="22" t="n">
+        <v>0.01128</v>
+      </c>
+      <c r="F25" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G25" s="23" t="n">
+        <v>0.01128</v>
+      </c>
+      <c r="H25" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="B26" s="22" t="n">
+        <v>0.00455</v>
+      </c>
+      <c r="C26" s="22" t="n">
+        <v>0.01469</v>
+      </c>
+      <c r="D26" s="22" t="n">
+        <v>0.01577</v>
+      </c>
+      <c r="E26" s="22" t="n">
+        <v>0.01577</v>
+      </c>
+      <c r="F26" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G26" s="23" t="n">
+        <v>0.01577</v>
+      </c>
+      <c r="H26" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="B27" s="22" t="n">
+        <v>0.00773</v>
+      </c>
+      <c r="C27" s="22" t="n">
+        <v>0.01313</v>
+      </c>
+      <c r="D27" s="22" t="n">
+        <v>0.01366</v>
+      </c>
+      <c r="E27" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F27" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G27" s="23" t="n">
+        <v>0.01386</v>
+      </c>
+      <c r="H27" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="B28" s="22" t="n">
+        <v>0.00494</v>
+      </c>
+      <c r="C28" s="22" t="n">
+        <v>0.00758</v>
+      </c>
+      <c r="D28" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E28" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F28" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G28" s="23" t="n">
+        <v>0.00906</v>
+      </c>
+      <c r="H28" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="B29" s="22" t="n">
+        <v>0.00215</v>
+      </c>
+      <c r="C29" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D29" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E29" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F29" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G29" s="23" t="n">
+        <v>0.00338</v>
+      </c>
+      <c r="H29" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30" ht="15" customHeight="1">
+      <c r="A30" s="21" t="inlineStr">
+        <is>
+          <t>How to read this table</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="44" customHeight="1">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>• Each cell is the part of the vintage's loss rate (principal ≥90 DPD today ÷ seasoned principal, ex-FPD — the same measure as the table above) that comes from accounts which had reached 90 days past due by the end of month n after the origination month. 'Today' is the full current loss rate. Cells are blank where month n has not yet ended.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="44" customHeight="1">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>• The loss on a vintage is essentially complete by month 4 on book: January–March 2026 show no further movement from month 4 to month 6–8. Because cash is applied to the oldest balances first, an account that defaults later has already repaid its earlier months' purchases, so late defaults fall on later vintages rather than reopening old ones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="44" customHeight="1">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>• Read across the 'Today' column for the trend in fully emerged vintages: 2.26% (Jan), 1.13% (Feb), 1.58% (Mar), 1.39% (Apr), 0.91% (May, at month 5 — effectively final). June is at month 4 with one month of emergence still to come.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="9">
     <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A30:H30"/>
     <mergeCell ref="A20:H20"/>
     <mergeCell ref="A16:H16"/>
     <mergeCell ref="A19:H19"/>
+    <mergeCell ref="A33:H33"/>
+    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="A31:H31"/>
     <mergeCell ref="A17:H17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2746,7 +3029,7 @@
       </c>
     </row>
     <row r="4" ht="75" customHeight="1">
-      <c r="A4" s="22" t="inlineStr">
+      <c r="A4" s="24" t="inlineStr">
         <is>
           <t>Scope</t>
         </is>
@@ -2758,7 +3041,7 @@
       </c>
     </row>
     <row r="5" ht="60" customHeight="1">
-      <c r="A5" s="22" t="inlineStr">
+      <c r="A5" s="24" t="inlineStr">
         <is>
           <t>Average receivables</t>
         </is>
@@ -2770,7 +3053,7 @@
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="A6" s="24" t="inlineStr">
         <is>
           <t>Annualization</t>
         </is>
@@ -2782,7 +3065,7 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="22" t="inlineStr">
+      <c r="A7" s="24" t="inlineStr">
         <is>
           <t>Revolving interest</t>
         </is>
@@ -2794,7 +3077,7 @@
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="A8" s="24" t="inlineStr">
         <is>
           <t>Installment interest and upfront fees</t>
         </is>
@@ -2806,7 +3089,7 @@
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="22" t="inlineStr">
+      <c r="A9" s="24" t="inlineStr">
         <is>
           <t>Late payment fees</t>
         </is>
@@ -2818,7 +3101,7 @@
       </c>
     </row>
     <row r="10" ht="90" customHeight="1">
-      <c r="A10" s="22" t="inlineStr">
+      <c r="A10" s="24" t="inlineStr">
         <is>
           <t>Interchange</t>
         </is>
@@ -2830,7 +3113,7 @@
       </c>
     </row>
     <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="22" t="inlineStr">
+      <c r="A11" s="24" t="inlineStr">
         <is>
           <t>Turnover</t>
         </is>
@@ -2842,7 +3125,7 @@
       </c>
     </row>
     <row r="12" ht="60" customHeight="1">
-      <c r="A12" s="22" t="inlineStr">
+      <c r="A12" s="24" t="inlineStr">
         <is>
           <t>Principal flow</t>
         </is>
@@ -2854,7 +3137,7 @@
       </c>
     </row>
     <row r="13" ht="90" customHeight="1">
-      <c r="A13" s="22" t="inlineStr">
+      <c r="A13" s="24" t="inlineStr">
         <is>
           <t>Principal originated (Loss Rate tab)</t>
         </is>
@@ -2866,7 +3149,7 @@
       </c>
     </row>
     <row r="14" ht="90" customHeight="1">
-      <c r="A14" s="22" t="inlineStr">
+      <c r="A14" s="24" t="inlineStr">
         <is>
           <t>Loss rate</t>
         </is>
@@ -2878,7 +3161,7 @@
       </c>
     </row>
     <row r="15" ht="45" customHeight="1">
-      <c r="A15" s="22" t="inlineStr">
+      <c r="A15" s="24" t="inlineStr">
         <is>
           <t>Loss on receivables</t>
         </is>
@@ -2890,7 +3173,7 @@
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="22" t="inlineStr">
+      <c r="A16" s="24" t="inlineStr">
         <is>
           <t>Net yield</t>
         </is>
@@ -2901,20 +3184,20 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="60" customHeight="1">
-      <c r="A17" s="22" t="inlineStr">
+    <row r="17" ht="75" customHeight="1">
+      <c r="A17" s="24" t="inlineStr">
         <is>
           <t>Sources</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Zed management reporting built from the i2c transaction and settlement extracts (revenue, receivables, purchase volume; as of 26 October 2026), the processor transaction feed (pay-a-friend transfers) and Zed's statement and delinquency data (originations, delinquency by origination month; as of 27 October 2026). September 2026 is the latest complete month.</t>
+          <t>Zed management reporting built from the i2c transaction and settlement extracts (revenue, receivables, purchase volume; as of 26 October 2026), the processor transaction feed (pay-a-friend transfers) and Zed's statement and delinquency data (originations, delinquency by origination month and delinquency history for the emergence table; as of 27 October 2026). September 2026 is the latest complete month.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="22" t="inlineStr">
+      <c r="A18" s="24" t="inlineStr">
         <is>
           <t>Prepared</t>
         </is>

</xml_diff>

<commit_message>
Portfolio Yield Analysis: Loss Rate column headers state role (seasoned / excluded / denominator / numerator); note row heights
</commit_message>
<xml_diff>
--- a/Prior Responses (outside data room)/Zed Portfolio Yield Analysis_20261027_DRAFT.xlsx
+++ b/Prior Responses (outside data room)/Zed Portfolio Yield Analysis_20261027_DRAFT.xlsx
@@ -2330,7 +2330,7 @@
       </c>
     </row>
     <row r="3"/>
-    <row r="4" ht="60" customHeight="1">
+    <row r="4" ht="75" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Origination month</t>
@@ -2348,27 +2348,27 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Principal on statements ≥90 days past due date (seasoned)</t>
+          <t>Of which seasoned: due date ≥90 days ago, so old enough to be measured</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Principal ≥90 DPD on first-payment-default accounts (excluded)</t>
+          <t>Excluded: principal 90+ DPD on first-payment-default accounts</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Seasoned principal, ex-FPD</t>
+          <t>Denominator: seasoned principal excluding FPD accounts</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Principal ≥90 DPD, ex-FPD</t>
+          <t>Numerator: principal 90+ DPD excluding FPD accounts</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Loss rate (≥90 DPD ex-FPD ÷ seasoned principal ex-FPD)</t>
+          <t>Loss rate = numerator ÷ denominator</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Portfolio Yield Analysis: shorter Loss Rate headers
</commit_message>
<xml_diff>
--- a/Prior Responses (outside data room)/Zed Portfolio Yield Analysis_20261027_DRAFT.xlsx
+++ b/Prior Responses (outside data room)/Zed Portfolio Yield Analysis_20261027_DRAFT.xlsx
@@ -2330,7 +2330,7 @@
       </c>
     </row>
     <row r="3"/>
-    <row r="4" ht="75" customHeight="1">
+    <row r="4" ht="48" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Origination month</t>
@@ -2338,7 +2338,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Accounts originating</t>
+          <t>Accounts</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -2348,27 +2348,27 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Of which seasoned: due date ≥90 days ago, so old enough to be measured</t>
+          <t>Seasoned principal (due ≥90 days ago)</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Excluded: principal 90+ DPD on first-payment-default accounts</t>
+          <t>Excluded: FPD principal 90+ DPD</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Denominator: seasoned principal excluding FPD accounts</t>
+          <t>Denominator: seasoned, ex-FPD</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Numerator: principal 90+ DPD excluding FPD accounts</t>
+          <t>Numerator: 90+ DPD, ex-FPD</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Loss rate = numerator ÷ denominator</t>
+          <t>Loss rate</t>
         </is>
       </c>
     </row>

</xml_diff>